<commit_message>
Update Excel template formatting and add Azure Functions configuration
</commit_message>
<xml_diff>
--- a/templates/Excel_templates/タイムシート(yyyy_mm).xlsx
+++ b/templates/Excel_templates/タイムシート(yyyy_mm).xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="28925"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29530"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\kenichi.yamamoto\Documents\wk_src\timesheet-api\templates\Excel_templates\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{84940733-89DA-40D6-A5EE-FD02FD04D2C5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7E086512-C782-410F-B9B1-6C9336D733E2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="MM月" sheetId="26" r:id="rId1"/>
@@ -42,7 +42,7 @@
 <sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="30" uniqueCount="27">
   <si>
     <t>月次タイムシート</t>
-    <phoneticPr fontId="3"/>
+    <phoneticPr fontId="2"/>
   </si>
   <si>
     <t>派遣就業場所</t>
@@ -55,7 +55,7 @@
     <rPh sb="4" eb="6">
       <t>バショ</t>
     </rPh>
-    <phoneticPr fontId="3"/>
+    <phoneticPr fontId="2"/>
   </si>
   <si>
     <t>名　称</t>
@@ -65,7 +65,7 @@
     <rPh sb="2" eb="3">
       <t>ショウ</t>
     </rPh>
-    <phoneticPr fontId="3"/>
+    <phoneticPr fontId="2"/>
   </si>
   <si>
     <t>出光興産株式会社</t>
@@ -78,7 +78,7 @@
     <rPh sb="4" eb="8">
       <t>カブ</t>
     </rPh>
-    <phoneticPr fontId="3"/>
+    <phoneticPr fontId="2"/>
   </si>
   <si>
     <t>就業場所</t>
@@ -88,7 +88,7 @@
     <rPh sb="2" eb="4">
       <t>バショ</t>
     </rPh>
-    <phoneticPr fontId="3"/>
+    <phoneticPr fontId="2"/>
   </si>
   <si>
     <t>部署名</t>
@@ -98,14 +98,14 @@
     <rPh sb="2" eb="3">
       <t>メイ</t>
     </rPh>
-    <phoneticPr fontId="3"/>
+    <phoneticPr fontId="2"/>
   </si>
   <si>
     <t>デジタル・ICT推進部</t>
     <rPh sb="8" eb="11">
       <t>スイシンブ</t>
     </rPh>
-    <phoneticPr fontId="3"/>
+    <phoneticPr fontId="2"/>
   </si>
   <si>
     <t>組織単位</t>
@@ -115,7 +115,7 @@
     <rPh sb="2" eb="4">
       <t>タンイ</t>
     </rPh>
-    <phoneticPr fontId="3"/>
+    <phoneticPr fontId="2"/>
   </si>
   <si>
     <t>派遣労働者氏名</t>
@@ -128,7 +128,7 @@
     <rPh sb="5" eb="7">
       <t>シメイ</t>
     </rPh>
-    <phoneticPr fontId="3"/>
+    <phoneticPr fontId="2"/>
   </si>
   <si>
     <t>氏　名</t>
@@ -138,11 +138,11 @@
     <rPh sb="2" eb="3">
       <t>ナ</t>
     </rPh>
-    <phoneticPr fontId="3"/>
+    <phoneticPr fontId="2"/>
   </si>
   <si>
     <t>アクセンチュア株式会社</t>
-    <phoneticPr fontId="3"/>
+    <phoneticPr fontId="2"/>
   </si>
   <si>
     <t>作業期間</t>
@@ -152,11 +152,11 @@
     <rPh sb="2" eb="4">
       <t>キカン</t>
     </rPh>
-    <phoneticPr fontId="3"/>
+    <phoneticPr fontId="2"/>
   </si>
   <si>
     <t>～</t>
-    <phoneticPr fontId="3"/>
+    <phoneticPr fontId="2"/>
   </si>
   <si>
     <t>責任の程度</t>
@@ -166,11 +166,11 @@
     <rPh sb="3" eb="5">
       <t>テイド</t>
     </rPh>
-    <phoneticPr fontId="3"/>
+    <phoneticPr fontId="2"/>
   </si>
   <si>
     <t>企画・運用担当者（役職、決裁権限は無し）</t>
-    <phoneticPr fontId="3"/>
+    <phoneticPr fontId="2"/>
   </si>
   <si>
     <t>日</t>
@@ -180,14 +180,14 @@
   </si>
   <si>
     <t>作業内容</t>
-    <phoneticPr fontId="3"/>
+    <phoneticPr fontId="2"/>
   </si>
   <si>
     <t>ACN業務</t>
     <rPh sb="3" eb="5">
       <t>ギョウム</t>
     </rPh>
-    <phoneticPr fontId="9"/>
+    <phoneticPr fontId="3"/>
   </si>
   <si>
     <t>始業時間</t>
@@ -203,14 +203,14 @@
     <rPh sb="2" eb="4">
       <t>ジカン</t>
     </rPh>
-    <phoneticPr fontId="3"/>
+    <phoneticPr fontId="2"/>
   </si>
   <si>
     <t>就業時間</t>
     <rPh sb="0" eb="2">
       <t>シュウギョウ</t>
     </rPh>
-    <phoneticPr fontId="3"/>
+    <phoneticPr fontId="2"/>
   </si>
   <si>
     <t>実働日</t>
@@ -226,11 +226,11 @@
     <rPh sb="2" eb="4">
       <t>ジカン</t>
     </rPh>
+    <phoneticPr fontId="2"/>
+  </si>
+  <si>
+    <t>東京都千代田区大手町一丁目 2 番 1 号</t>
     <phoneticPr fontId="3"/>
-  </si>
-  <si>
-    <t>東京都千代田区大手町一丁目 2 番 1 号</t>
-    <phoneticPr fontId="9"/>
   </si>
 </sst>
 </file>
@@ -255,46 +255,8 @@
       <charset val="128"/>
     </font>
     <font>
-      <b/>
-      <sz val="16"/>
-      <name val="メイリオ"/>
-      <family val="3"/>
-      <charset val="128"/>
-    </font>
-    <font>
       <sz val="6"/>
       <name val="ＭＳ Ｐゴシック"/>
-      <family val="3"/>
-      <charset val="128"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="メイリオ"/>
-      <family val="3"/>
-      <charset val="128"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="11"/>
-      <name val="メイリオ"/>
-      <family val="3"/>
-      <charset val="128"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <name val="メイリオ"/>
-      <family val="3"/>
-      <charset val="128"/>
-    </font>
-    <font>
-      <sz val="9"/>
-      <name val="メイリオ"/>
-      <family val="3"/>
-      <charset val="128"/>
-    </font>
-    <font>
-      <sz val="12"/>
-      <name val="メイリオ"/>
       <family val="3"/>
       <charset val="128"/>
     </font>
@@ -309,6 +271,44 @@
       <color theme="1"/>
       <name val="Arial"/>
       <family val="2"/>
+      <charset val="128"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="16"/>
+      <name val="Meiryo UI"/>
+      <family val="3"/>
+      <charset val="128"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Meiryo UI"/>
+      <family val="3"/>
+      <charset val="128"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <name val="Meiryo UI"/>
+      <family val="3"/>
+      <charset val="128"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Meiryo UI"/>
+      <family val="3"/>
+      <charset val="128"/>
+    </font>
+    <font>
+      <sz val="9"/>
+      <name val="Meiryo UI"/>
+      <family val="3"/>
+      <charset val="128"/>
+    </font>
+    <font>
+      <sz val="12"/>
+      <name val="Meiryo UI"/>
+      <family val="3"/>
       <charset val="128"/>
     </font>
   </fonts>
@@ -497,7 +497,7 @@
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
-    <xf numFmtId="38" fontId="10" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="38" fontId="4" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
@@ -505,197 +505,197 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="49" fontId="2" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="5" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="centerContinuous" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="centerContinuous" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="49" fontId="6" fillId="0" borderId="10" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="14" fontId="6" fillId="0" borderId="10" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="20" fontId="4" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="7" fillId="3" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="7" fillId="3" borderId="2" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="7" fillId="3" borderId="3" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="14" fontId="6" fillId="0" borderId="4" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="14" fontId="6" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="3" borderId="5" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="3" borderId="6" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="3" borderId="7" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="1" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="2" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="3" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="3" borderId="4" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="3" borderId="0" xfId="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="3" borderId="8" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="1" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="2" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="3" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="3" borderId="9" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="3" borderId="10" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="3" borderId="11" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="8" fillId="3" borderId="5" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="8" fillId="3" borderId="6" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="8" fillId="3" borderId="7" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="4" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="8" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="1" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="2" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="3" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="8" fillId="3" borderId="4" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="8" fillId="3" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="8" fillId="3" borderId="8" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="14" fontId="8" fillId="4" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="14" fontId="8" fillId="4" borderId="2" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="2" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="14" fontId="8" fillId="4" borderId="3" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="8" fillId="0" borderId="10" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="14" fontId="8" fillId="0" borderId="10" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="6" fillId="2" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="centerContinuous" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="centerContinuous" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="2" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="centerContinuous" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="2" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="centerContinuous" vertical="center" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="12" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="centerContinuous" vertical="center"/>
+    </xf>
+    <xf numFmtId="176" fontId="6" fillId="0" borderId="9" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="9" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="centerContinuous" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="9" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="176" fontId="4" fillId="0" borderId="9" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="20" fontId="8" fillId="0" borderId="9" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="2" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="20" fontId="8" fillId="0" borderId="13" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="20" fontId="10" fillId="0" borderId="9" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="9" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="20" fontId="10" fillId="0" borderId="13" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="9" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="centerContinuous" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="2" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="20" fontId="6" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="2" fontId="8" fillId="0" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="6" fillId="0" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="6" fillId="0" borderId="3" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="38" fontId="10" fillId="0" borderId="1" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="3" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="2" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="49" fontId="4" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="20" fontId="10" fillId="0" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="3" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="38" fontId="8" fillId="0" borderId="1" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="2" fontId="10" fillId="0" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="2" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="3" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="49" fontId="4" fillId="2" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="centerContinuous" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="centerContinuous" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="2" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="centerContinuous" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="2" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="centerContinuous" vertical="center" shrinkToFit="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="12" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="centerContinuous" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="2" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="20" fontId="8" fillId="0" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="6" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="2" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="4" fillId="0" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="4" fillId="0" borderId="3" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="3" borderId="4" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="3" borderId="0" xfId="1" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="3" borderId="8" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="2" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="3" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="3" borderId="9" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="3" borderId="10" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="3" borderId="11" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="5" fillId="3" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="5" fillId="3" borderId="2" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="5" fillId="3" borderId="3" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="6" fillId="3" borderId="5" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="6" fillId="3" borderId="6" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="6" fillId="3" borderId="7" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="4" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="8" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="2" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="3" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="6" fillId="3" borderId="4" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="6" fillId="3" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="6" fillId="3" borderId="8" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="14" fontId="6" fillId="4" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="14" fontId="6" fillId="4" borderId="2" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="14" fontId="6" fillId="4" borderId="3" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="14" fontId="4" fillId="0" borderId="4" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="14" fontId="4" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="3" borderId="5" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="3" borderId="6" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="3" borderId="7" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="2" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="3" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="3" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="2" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="3">
@@ -983,20 +983,20 @@
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="A1:M44"/>
-  <sheetFormatPr defaultColWidth="7.25" defaultRowHeight="18.75" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultColWidth="7.26953125" defaultRowHeight="15" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="3.125" style="16" customWidth="1"/>
-    <col min="2" max="2" width="3.125" style="3" customWidth="1"/>
-    <col min="3" max="3" width="7.5" style="3" customWidth="1"/>
-    <col min="4" max="7" width="8.125" style="3" customWidth="1"/>
-    <col min="8" max="8" width="7.5" style="3" bestFit="1" customWidth="1"/>
-    <col min="9" max="10" width="7.5" style="3" customWidth="1"/>
-    <col min="11" max="11" width="7.5" style="3" bestFit="1" customWidth="1"/>
-    <col min="12" max="14" width="7.25" style="3" customWidth="1"/>
-    <col min="15" max="16384" width="7.25" style="3"/>
+    <col min="1" max="1" width="3.08984375" style="62" customWidth="1"/>
+    <col min="2" max="2" width="3.08984375" style="3" customWidth="1"/>
+    <col min="3" max="3" width="7.453125" style="3" customWidth="1"/>
+    <col min="4" max="7" width="8.08984375" style="3" customWidth="1"/>
+    <col min="8" max="8" width="7.453125" style="3" bestFit="1" customWidth="1"/>
+    <col min="9" max="10" width="7.453125" style="3" customWidth="1"/>
+    <col min="11" max="11" width="7.453125" style="3" bestFit="1" customWidth="1"/>
+    <col min="12" max="14" width="7.26953125" style="3" customWidth="1"/>
+    <col min="15" max="16384" width="7.26953125" style="3"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:13" ht="25.35" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:13" ht="25.35" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1011,831 +1011,825 @@
       <c r="J1" s="2"/>
       <c r="K1" s="2"/>
     </row>
-    <row r="2" spans="1:13" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="40" t="s">
+    <row r="2" spans="1:13" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A2" s="4" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="41"/>
-      <c r="C2" s="41"/>
-      <c r="D2" s="41"/>
-      <c r="E2" s="41"/>
-      <c r="F2" s="41"/>
-      <c r="G2" s="41"/>
-      <c r="H2" s="42"/>
-      <c r="I2" s="57">
+      <c r="B2" s="5"/>
+      <c r="C2" s="5"/>
+      <c r="D2" s="5"/>
+      <c r="E2" s="5"/>
+      <c r="F2" s="5"/>
+      <c r="G2" s="5"/>
+      <c r="H2" s="6"/>
+      <c r="I2" s="7">
         <f>G9+1</f>
         <v>1</v>
       </c>
-      <c r="J2" s="58"/>
-      <c r="K2" s="58"/>
-    </row>
-    <row r="3" spans="1:13" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A3" s="59" t="s">
+      <c r="J2" s="8"/>
+      <c r="K2" s="8"/>
+    </row>
+    <row r="3" spans="1:13" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A3" s="9" t="s">
         <v>2</v>
       </c>
-      <c r="B3" s="60"/>
-      <c r="C3" s="61"/>
-      <c r="D3" s="62" t="s">
+      <c r="B3" s="10"/>
+      <c r="C3" s="11"/>
+      <c r="D3" s="12" t="s">
         <v>3</v>
       </c>
-      <c r="E3" s="63"/>
-      <c r="F3" s="63"/>
-      <c r="G3" s="63"/>
-      <c r="H3" s="64"/>
-    </row>
-    <row r="4" spans="1:13" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A4" s="31" t="s">
+      <c r="E3" s="13"/>
+      <c r="F3" s="13"/>
+      <c r="G3" s="13"/>
+      <c r="H3" s="14"/>
+    </row>
+    <row r="4" spans="1:13" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A4" s="15" t="s">
         <v>4</v>
       </c>
-      <c r="B4" s="32"/>
-      <c r="C4" s="33"/>
-      <c r="D4" s="34" t="s">
+      <c r="B4" s="16"/>
+      <c r="C4" s="17"/>
+      <c r="D4" s="18" t="s">
         <v>26</v>
       </c>
-      <c r="E4" s="35"/>
-      <c r="F4" s="35"/>
-      <c r="G4" s="35"/>
-      <c r="H4" s="36"/>
-    </row>
-    <row r="5" spans="1:13" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A5" s="31" t="s">
+      <c r="E4" s="19"/>
+      <c r="F4" s="19"/>
+      <c r="G4" s="19"/>
+      <c r="H4" s="20"/>
+    </row>
+    <row r="5" spans="1:13" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A5" s="15" t="s">
         <v>5</v>
       </c>
-      <c r="B5" s="32"/>
-      <c r="C5" s="33"/>
-      <c r="D5" s="34" t="s">
+      <c r="B5" s="16"/>
+      <c r="C5" s="17"/>
+      <c r="D5" s="18" t="s">
         <v>6</v>
       </c>
-      <c r="E5" s="35"/>
-      <c r="F5" s="35"/>
-      <c r="G5" s="35"/>
-      <c r="H5" s="36"/>
-    </row>
-    <row r="6" spans="1:13" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A6" s="37" t="s">
+      <c r="E5" s="19"/>
+      <c r="F5" s="19"/>
+      <c r="G5" s="19"/>
+      <c r="H5" s="20"/>
+    </row>
+    <row r="6" spans="1:13" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A6" s="21" t="s">
         <v>7</v>
       </c>
-      <c r="B6" s="38"/>
-      <c r="C6" s="39"/>
-      <c r="D6" s="34"/>
-      <c r="E6" s="35"/>
-      <c r="F6" s="35"/>
-      <c r="G6" s="35"/>
-      <c r="H6" s="36"/>
-    </row>
-    <row r="7" spans="1:13" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A7" s="40" t="s">
+      <c r="B6" s="22"/>
+      <c r="C6" s="23"/>
+      <c r="D6" s="18"/>
+      <c r="E6" s="19"/>
+      <c r="F6" s="19"/>
+      <c r="G6" s="19"/>
+      <c r="H6" s="20"/>
+    </row>
+    <row r="7" spans="1:13" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A7" s="4" t="s">
         <v>8</v>
       </c>
-      <c r="B7" s="41"/>
-      <c r="C7" s="41"/>
-      <c r="D7" s="41"/>
-      <c r="E7" s="41"/>
-      <c r="F7" s="41"/>
-      <c r="G7" s="41"/>
-      <c r="H7" s="42"/>
-    </row>
-    <row r="8" spans="1:13" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A8" s="43" t="s">
+      <c r="B7" s="5"/>
+      <c r="C7" s="5"/>
+      <c r="D7" s="5"/>
+      <c r="E7" s="5"/>
+      <c r="F7" s="5"/>
+      <c r="G7" s="5"/>
+      <c r="H7" s="6"/>
+    </row>
+    <row r="8" spans="1:13" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A8" s="24" t="s">
         <v>9</v>
       </c>
-      <c r="B8" s="44"/>
-      <c r="C8" s="45"/>
-      <c r="D8" s="46"/>
-      <c r="E8" s="47"/>
-      <c r="F8" s="48" t="s">
+      <c r="B8" s="25"/>
+      <c r="C8" s="26"/>
+      <c r="D8" s="27"/>
+      <c r="E8" s="28"/>
+      <c r="F8" s="29" t="s">
         <v>10</v>
       </c>
-      <c r="G8" s="49"/>
-      <c r="H8" s="50"/>
-    </row>
-    <row r="9" spans="1:13" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A9" s="51" t="s">
+      <c r="G8" s="30"/>
+      <c r="H8" s="31"/>
+    </row>
+    <row r="9" spans="1:13" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A9" s="32" t="s">
         <v>11</v>
       </c>
-      <c r="B9" s="52"/>
-      <c r="C9" s="53"/>
-      <c r="D9" s="54"/>
-      <c r="E9" s="55"/>
-      <c r="F9" s="26" t="s">
+      <c r="B9" s="33"/>
+      <c r="C9" s="34"/>
+      <c r="D9" s="35"/>
+      <c r="E9" s="36"/>
+      <c r="F9" s="37" t="s">
         <v>12</v>
       </c>
-      <c r="G9" s="55"/>
-      <c r="H9" s="56"/>
-    </row>
-    <row r="10" spans="1:13" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A10" s="37" t="s">
+      <c r="G9" s="36"/>
+      <c r="H9" s="38"/>
+    </row>
+    <row r="10" spans="1:13" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A10" s="21" t="s">
         <v>13</v>
       </c>
-      <c r="B10" s="38"/>
-      <c r="C10" s="39"/>
-      <c r="D10" s="34" t="s">
+      <c r="B10" s="22"/>
+      <c r="C10" s="23"/>
+      <c r="D10" s="18" t="s">
         <v>14</v>
       </c>
-      <c r="E10" s="35"/>
-      <c r="F10" s="35"/>
-      <c r="G10" s="35"/>
-      <c r="H10" s="36"/>
-    </row>
-    <row r="11" spans="1:13" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A11" s="4"/>
-      <c r="B11" s="4"/>
-      <c r="C11" s="5"/>
-      <c r="D11" s="5"/>
-      <c r="E11" s="6"/>
-      <c r="F11" s="5"/>
-      <c r="G11" s="5"/>
-    </row>
-    <row r="12" spans="1:13" ht="19.350000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A12" s="21" t="s">
+      <c r="E10" s="19"/>
+      <c r="F10" s="19"/>
+      <c r="G10" s="19"/>
+      <c r="H10" s="20"/>
+    </row>
+    <row r="11" spans="1:13" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A11" s="39"/>
+      <c r="B11" s="39"/>
+      <c r="C11" s="40"/>
+      <c r="D11" s="40"/>
+      <c r="E11" s="41"/>
+      <c r="F11" s="40"/>
+      <c r="G11" s="40"/>
+    </row>
+    <row r="12" spans="1:13" ht="19.350000000000001" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A12" s="42" t="s">
         <v>15</v>
       </c>
-      <c r="B12" s="22" t="s">
+      <c r="B12" s="43" t="s">
         <v>16</v>
       </c>
-      <c r="C12" s="22" t="s">
+      <c r="C12" s="43" t="s">
         <v>17</v>
       </c>
-      <c r="D12" s="23"/>
-      <c r="E12" s="23"/>
-      <c r="F12" s="23"/>
-      <c r="G12" s="24" t="s">
+      <c r="D12" s="44"/>
+      <c r="E12" s="44"/>
+      <c r="F12" s="44"/>
+      <c r="G12" s="45" t="s">
         <v>18</v>
       </c>
-      <c r="H12" s="22" t="s">
+      <c r="H12" s="43" t="s">
         <v>19</v>
       </c>
-      <c r="I12" s="22" t="s">
+      <c r="I12" s="43" t="s">
         <v>20</v>
       </c>
-      <c r="J12" s="25" t="s">
+      <c r="J12" s="46" t="s">
         <v>21</v>
       </c>
-      <c r="K12" s="25" t="s">
+      <c r="K12" s="46" t="s">
         <v>22</v>
       </c>
     </row>
-    <row r="13" spans="1:13" ht="19.350000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A13" s="8">
+    <row r="13" spans="1:13" ht="19.350000000000001" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A13" s="47">
         <f>D9</f>
         <v>0</v>
       </c>
-      <c r="B13" s="12" t="str">
+      <c r="B13" s="48" t="str">
         <f>IF(A13="","",CHOOSE(WEEKDAY(A13),"日","月","火","水","木","金","土"))</f>
         <v>土</v>
       </c>
-      <c r="C13" s="11"/>
-      <c r="D13" s="20"/>
-      <c r="E13" s="20"/>
-      <c r="F13" s="20"/>
-      <c r="G13" s="17"/>
-      <c r="H13" s="9"/>
-      <c r="I13" s="9"/>
-      <c r="J13" s="10"/>
-      <c r="K13" s="10"/>
-      <c r="M13" s="7"/>
-    </row>
-    <row r="14" spans="1:13" ht="19.350000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A14" s="8">
+      <c r="C13" s="49"/>
+      <c r="D13" s="50"/>
+      <c r="E13" s="50"/>
+      <c r="F13" s="50"/>
+      <c r="G13" s="63"/>
+      <c r="H13" s="51"/>
+      <c r="I13" s="51"/>
+      <c r="J13" s="52"/>
+      <c r="K13" s="52"/>
+      <c r="M13" s="53"/>
+    </row>
+    <row r="14" spans="1:13" ht="19.350000000000001" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A14" s="47">
         <f>A13+1</f>
         <v>1</v>
       </c>
-      <c r="B14" s="12" t="str">
+      <c r="B14" s="48" t="str">
         <f t="shared" ref="B14:B20" si="0">IF(A14="","",CHOOSE(WEEKDAY(A14),"日","月","火","水","木","金","土"))</f>
         <v>日</v>
       </c>
-      <c r="C14" s="11"/>
-      <c r="D14" s="20"/>
-      <c r="E14" s="20"/>
-      <c r="F14" s="20"/>
-      <c r="G14" s="17"/>
-      <c r="H14" s="9"/>
-      <c r="I14" s="9"/>
-      <c r="J14" s="10"/>
-      <c r="K14" s="10"/>
-      <c r="M14" s="7"/>
-    </row>
-    <row r="15" spans="1:13" ht="19.350000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A15" s="8">
+      <c r="C14" s="49"/>
+      <c r="D14" s="50"/>
+      <c r="E14" s="50"/>
+      <c r="F14" s="50"/>
+      <c r="G14" s="63"/>
+      <c r="H14" s="51"/>
+      <c r="I14" s="51"/>
+      <c r="J14" s="52"/>
+      <c r="K14" s="52"/>
+      <c r="M14" s="53"/>
+    </row>
+    <row r="15" spans="1:13" ht="19.350000000000001" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A15" s="47">
         <f>A14+1</f>
         <v>2</v>
       </c>
-      <c r="B15" s="12" t="str">
+      <c r="B15" s="48" t="str">
         <f t="shared" si="0"/>
         <v>月</v>
       </c>
-      <c r="C15" s="11"/>
-      <c r="D15" s="20"/>
-      <c r="E15" s="20"/>
-      <c r="F15" s="20"/>
-      <c r="G15" s="17"/>
-      <c r="H15" s="9"/>
-      <c r="I15" s="9"/>
-      <c r="J15" s="10"/>
-      <c r="K15" s="10"/>
-      <c r="M15" s="7"/>
-    </row>
-    <row r="16" spans="1:13" ht="19.350000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A16" s="8">
+      <c r="C15" s="49"/>
+      <c r="D15" s="50"/>
+      <c r="E15" s="50"/>
+      <c r="F15" s="50"/>
+      <c r="G15" s="63"/>
+      <c r="H15" s="51"/>
+      <c r="I15" s="51"/>
+      <c r="J15" s="52"/>
+      <c r="K15" s="52"/>
+      <c r="M15" s="53"/>
+    </row>
+    <row r="16" spans="1:13" ht="19.350000000000001" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A16" s="47">
         <f>A15+1</f>
         <v>3</v>
       </c>
-      <c r="B16" s="12" t="str">
+      <c r="B16" s="48" t="str">
         <f t="shared" si="0"/>
         <v>火</v>
       </c>
-      <c r="C16" s="11"/>
-      <c r="D16" s="20"/>
-      <c r="E16" s="20"/>
-      <c r="F16" s="20"/>
-      <c r="G16" s="17"/>
-      <c r="H16" s="9"/>
-      <c r="I16" s="9"/>
-      <c r="J16" s="10"/>
-      <c r="K16" s="10"/>
-      <c r="M16" s="7"/>
-    </row>
-    <row r="17" spans="1:13" ht="19.350000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A17" s="8">
+      <c r="C16" s="49"/>
+      <c r="D16" s="50"/>
+      <c r="E16" s="50"/>
+      <c r="F16" s="50"/>
+      <c r="G16" s="63"/>
+      <c r="H16" s="51"/>
+      <c r="I16" s="51"/>
+      <c r="J16" s="52"/>
+      <c r="K16" s="52"/>
+      <c r="M16" s="53"/>
+    </row>
+    <row r="17" spans="1:13" ht="19.350000000000001" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A17" s="47">
         <f>A16+1</f>
         <v>4</v>
       </c>
-      <c r="B17" s="12" t="str">
+      <c r="B17" s="48" t="str">
         <f t="shared" si="0"/>
         <v>水</v>
       </c>
-      <c r="C17" s="11"/>
-      <c r="D17" s="20"/>
-      <c r="E17" s="20"/>
-      <c r="F17" s="20"/>
-      <c r="G17" s="17"/>
-      <c r="H17" s="9"/>
-      <c r="I17" s="9"/>
-      <c r="J17" s="10"/>
-      <c r="K17" s="10"/>
-      <c r="M17" s="7"/>
-    </row>
-    <row r="18" spans="1:13" ht="19.350000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A18" s="8">
+      <c r="C17" s="49"/>
+      <c r="D17" s="50"/>
+      <c r="E17" s="50"/>
+      <c r="F17" s="50"/>
+      <c r="G17" s="63"/>
+      <c r="H17" s="51"/>
+      <c r="I17" s="51"/>
+      <c r="J17" s="52"/>
+      <c r="K17" s="52"/>
+      <c r="M17" s="53"/>
+    </row>
+    <row r="18" spans="1:13" ht="19.350000000000001" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A18" s="47">
         <f>A17+1</f>
         <v>5</v>
       </c>
-      <c r="B18" s="12" t="str">
+      <c r="B18" s="48" t="str">
         <f t="shared" si="0"/>
         <v>木</v>
       </c>
-      <c r="C18" s="11"/>
-      <c r="D18" s="20"/>
-      <c r="E18" s="20"/>
-      <c r="F18" s="20"/>
-      <c r="G18" s="17"/>
-      <c r="H18" s="9"/>
-      <c r="I18" s="9"/>
-      <c r="J18" s="10"/>
-      <c r="K18" s="10"/>
-      <c r="M18" s="7"/>
-    </row>
-    <row r="19" spans="1:13" ht="19.350000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A19" s="8">
+      <c r="C18" s="49"/>
+      <c r="D18" s="50"/>
+      <c r="E18" s="50"/>
+      <c r="F18" s="50"/>
+      <c r="G18" s="63"/>
+      <c r="H18" s="51"/>
+      <c r="I18" s="51"/>
+      <c r="J18" s="52"/>
+      <c r="K18" s="52"/>
+      <c r="M18" s="53"/>
+    </row>
+    <row r="19" spans="1:13" ht="19.350000000000001" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A19" s="47">
         <f t="shared" ref="A19:A20" si="1">A18+1</f>
         <v>6</v>
       </c>
-      <c r="B19" s="12" t="str">
+      <c r="B19" s="48" t="str">
         <f t="shared" si="0"/>
         <v>金</v>
       </c>
-      <c r="C19" s="11"/>
-      <c r="D19" s="20"/>
-      <c r="E19" s="20"/>
-      <c r="F19" s="20"/>
-      <c r="G19" s="17"/>
-      <c r="H19" s="9"/>
-      <c r="I19" s="9"/>
-      <c r="J19" s="10"/>
-      <c r="K19" s="10"/>
-      <c r="M19" s="7"/>
-    </row>
-    <row r="20" spans="1:13" ht="19.350000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A20" s="8">
+      <c r="C19" s="49"/>
+      <c r="D19" s="50"/>
+      <c r="E19" s="50"/>
+      <c r="F19" s="50"/>
+      <c r="G19" s="63"/>
+      <c r="H19" s="51"/>
+      <c r="I19" s="51"/>
+      <c r="J19" s="52"/>
+      <c r="K19" s="52"/>
+      <c r="M19" s="53"/>
+    </row>
+    <row r="20" spans="1:13" ht="19.350000000000001" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A20" s="47">
         <f t="shared" si="1"/>
         <v>7</v>
       </c>
-      <c r="B20" s="12" t="str">
+      <c r="B20" s="48" t="str">
         <f t="shared" si="0"/>
         <v>土</v>
       </c>
-      <c r="C20" s="11"/>
-      <c r="D20" s="20"/>
-      <c r="E20" s="20"/>
-      <c r="F20" s="20"/>
-      <c r="G20" s="17"/>
-      <c r="H20" s="9"/>
-      <c r="I20" s="9"/>
-      <c r="J20" s="10"/>
-      <c r="K20" s="10"/>
-      <c r="M20" s="7"/>
-    </row>
-    <row r="21" spans="1:13" ht="19.350000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A21" s="8">
+      <c r="C20" s="49"/>
+      <c r="D20" s="50"/>
+      <c r="E20" s="50"/>
+      <c r="F20" s="50"/>
+      <c r="G20" s="63"/>
+      <c r="H20" s="51"/>
+      <c r="I20" s="51"/>
+      <c r="J20" s="52"/>
+      <c r="K20" s="52"/>
+      <c r="M20" s="53"/>
+    </row>
+    <row r="21" spans="1:13" ht="19.350000000000001" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A21" s="47">
         <f>A20+1</f>
         <v>8</v>
       </c>
-      <c r="B21" s="12" t="str">
+      <c r="B21" s="48" t="str">
         <f t="shared" ref="B21:B27" si="2">IF(A21="","",CHOOSE(WEEKDAY(A21),"日","月","火","水","木","金","土"))</f>
         <v>日</v>
       </c>
-      <c r="C21" s="11"/>
-      <c r="D21" s="20"/>
-      <c r="E21" s="20"/>
-      <c r="F21" s="20"/>
-      <c r="G21" s="17"/>
-      <c r="H21" s="9"/>
-      <c r="I21" s="9"/>
-      <c r="J21" s="10"/>
-      <c r="K21" s="10"/>
-      <c r="M21" s="7"/>
-    </row>
-    <row r="22" spans="1:13" ht="19.350000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A22" s="8">
+      <c r="C21" s="49"/>
+      <c r="D21" s="50"/>
+      <c r="E21" s="50"/>
+      <c r="F21" s="50"/>
+      <c r="G21" s="63"/>
+      <c r="H21" s="51"/>
+      <c r="I21" s="51"/>
+      <c r="J21" s="52"/>
+      <c r="K21" s="52"/>
+      <c r="M21" s="53"/>
+    </row>
+    <row r="22" spans="1:13" ht="19.350000000000001" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A22" s="47">
         <f>A21+1</f>
         <v>9</v>
       </c>
-      <c r="B22" s="12" t="str">
+      <c r="B22" s="48" t="str">
         <f t="shared" si="2"/>
         <v>月</v>
       </c>
-      <c r="C22" s="11"/>
-      <c r="D22" s="20"/>
-      <c r="E22" s="20"/>
-      <c r="F22" s="20"/>
-      <c r="G22" s="17"/>
-      <c r="H22" s="9"/>
-      <c r="I22" s="9"/>
-      <c r="J22" s="10"/>
-      <c r="K22" s="10"/>
-      <c r="M22" s="7"/>
-    </row>
-    <row r="23" spans="1:13" ht="19.350000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A23" s="8">
+      <c r="C22" s="49"/>
+      <c r="D22" s="50"/>
+      <c r="E22" s="50"/>
+      <c r="F22" s="50"/>
+      <c r="G22" s="63"/>
+      <c r="H22" s="51"/>
+      <c r="I22" s="51"/>
+      <c r="J22" s="52"/>
+      <c r="K22" s="52"/>
+      <c r="M22" s="53"/>
+    </row>
+    <row r="23" spans="1:13" ht="19.350000000000001" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A23" s="47">
         <f>A22+1</f>
         <v>10</v>
       </c>
-      <c r="B23" s="12" t="str">
+      <c r="B23" s="48" t="str">
         <f t="shared" si="2"/>
         <v>火</v>
       </c>
-      <c r="C23" s="11"/>
-      <c r="D23" s="20"/>
-      <c r="E23" s="20"/>
-      <c r="F23" s="20"/>
-      <c r="G23" s="17"/>
-      <c r="H23" s="9"/>
-      <c r="I23" s="9"/>
-      <c r="J23" s="10"/>
-      <c r="K23" s="10"/>
-      <c r="M23" s="7"/>
-    </row>
-    <row r="24" spans="1:13" ht="19.350000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A24" s="8">
+      <c r="C23" s="49"/>
+      <c r="D23" s="50"/>
+      <c r="E23" s="50"/>
+      <c r="F23" s="50"/>
+      <c r="G23" s="63"/>
+      <c r="H23" s="51"/>
+      <c r="I23" s="51"/>
+      <c r="J23" s="52"/>
+      <c r="K23" s="52"/>
+      <c r="M23" s="53"/>
+    </row>
+    <row r="24" spans="1:13" ht="19.350000000000001" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A24" s="47">
         <f>A23+1</f>
         <v>11</v>
       </c>
-      <c r="B24" s="12" t="str">
+      <c r="B24" s="48" t="str">
         <f t="shared" si="2"/>
         <v>水</v>
       </c>
-      <c r="C24" s="11"/>
-      <c r="D24" s="20"/>
-      <c r="E24" s="20"/>
-      <c r="F24" s="20"/>
-      <c r="G24" s="17"/>
-      <c r="H24" s="9"/>
-      <c r="I24" s="9"/>
-      <c r="J24" s="10"/>
-      <c r="K24" s="10"/>
-      <c r="M24" s="7"/>
-    </row>
-    <row r="25" spans="1:13" ht="19.350000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A25" s="8">
+      <c r="C24" s="49"/>
+      <c r="D24" s="50"/>
+      <c r="E24" s="50"/>
+      <c r="F24" s="50"/>
+      <c r="G24" s="63"/>
+      <c r="H24" s="51"/>
+      <c r="I24" s="51"/>
+      <c r="J24" s="52"/>
+      <c r="K24" s="52"/>
+      <c r="M24" s="53"/>
+    </row>
+    <row r="25" spans="1:13" ht="19.350000000000001" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A25" s="47">
         <f>A24+1</f>
         <v>12</v>
       </c>
-      <c r="B25" s="12" t="str">
+      <c r="B25" s="48" t="str">
         <f t="shared" si="2"/>
         <v>木</v>
       </c>
-      <c r="C25" s="11"/>
-      <c r="D25" s="20"/>
-      <c r="E25" s="20"/>
-      <c r="F25" s="20"/>
-      <c r="G25" s="17"/>
-      <c r="H25" s="9"/>
-      <c r="I25" s="9"/>
-      <c r="J25" s="10"/>
-      <c r="K25" s="10"/>
-      <c r="M25" s="7"/>
-    </row>
-    <row r="26" spans="1:13" ht="19.350000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A26" s="8">
+      <c r="C25" s="49"/>
+      <c r="D25" s="50"/>
+      <c r="E25" s="50"/>
+      <c r="F25" s="50"/>
+      <c r="G25" s="63"/>
+      <c r="H25" s="51"/>
+      <c r="I25" s="51"/>
+      <c r="J25" s="52"/>
+      <c r="K25" s="52"/>
+      <c r="M25" s="53"/>
+    </row>
+    <row r="26" spans="1:13" ht="19.350000000000001" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A26" s="47">
         <f t="shared" ref="A26:A31" si="3">A25+1</f>
         <v>13</v>
       </c>
-      <c r="B26" s="12" t="str">
+      <c r="B26" s="48" t="str">
         <f t="shared" si="2"/>
         <v>金</v>
       </c>
-      <c r="C26" s="11"/>
-      <c r="D26" s="20"/>
-      <c r="E26" s="20"/>
-      <c r="F26" s="20"/>
-      <c r="G26" s="17"/>
-      <c r="H26" s="9"/>
-      <c r="I26" s="9"/>
-      <c r="J26" s="10"/>
-      <c r="K26" s="10"/>
-      <c r="M26" s="7"/>
-    </row>
-    <row r="27" spans="1:13" ht="19.350000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A27" s="8">
+      <c r="C26" s="49"/>
+      <c r="D26" s="50"/>
+      <c r="E26" s="50"/>
+      <c r="F26" s="50"/>
+      <c r="G26" s="63"/>
+      <c r="H26" s="51"/>
+      <c r="I26" s="51"/>
+      <c r="J26" s="52"/>
+      <c r="K26" s="52"/>
+      <c r="M26" s="53"/>
+    </row>
+    <row r="27" spans="1:13" ht="19.350000000000001" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A27" s="47">
         <f t="shared" si="3"/>
         <v>14</v>
       </c>
-      <c r="B27" s="12" t="str">
+      <c r="B27" s="48" t="str">
         <f t="shared" si="2"/>
         <v>土</v>
       </c>
-      <c r="C27" s="11"/>
-      <c r="D27" s="20"/>
-      <c r="E27" s="20"/>
-      <c r="F27" s="20"/>
-      <c r="G27" s="17"/>
-      <c r="H27" s="9"/>
-      <c r="I27" s="9"/>
-      <c r="J27" s="10"/>
-      <c r="K27" s="10"/>
-      <c r="M27" s="7"/>
-    </row>
-    <row r="28" spans="1:13" ht="19.350000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A28" s="8">
+      <c r="C27" s="49"/>
+      <c r="D27" s="50"/>
+      <c r="E27" s="50"/>
+      <c r="F27" s="50"/>
+      <c r="G27" s="63"/>
+      <c r="H27" s="51"/>
+      <c r="I27" s="51"/>
+      <c r="J27" s="52"/>
+      <c r="K27" s="52"/>
+      <c r="M27" s="53"/>
+    </row>
+    <row r="28" spans="1:13" ht="19.350000000000001" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A28" s="47">
         <f t="shared" si="3"/>
         <v>15</v>
       </c>
-      <c r="B28" s="12" t="str">
+      <c r="B28" s="48" t="str">
         <f>IF(A28="","",CHOOSE(WEEKDAY(A28),"日","月","火","水","木","金","土"))</f>
         <v>日</v>
       </c>
-      <c r="C28" s="11"/>
-      <c r="D28" s="20"/>
-      <c r="E28" s="20"/>
-      <c r="F28" s="20"/>
-      <c r="G28" s="17"/>
-      <c r="H28" s="9"/>
-      <c r="I28" s="9"/>
-      <c r="J28" s="10"/>
-      <c r="K28" s="10"/>
-      <c r="M28" s="7"/>
-    </row>
-    <row r="29" spans="1:13" ht="19.350000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A29" s="8">
+      <c r="C28" s="49"/>
+      <c r="D28" s="50"/>
+      <c r="E28" s="50"/>
+      <c r="F28" s="50"/>
+      <c r="G28" s="63"/>
+      <c r="H28" s="51"/>
+      <c r="I28" s="51"/>
+      <c r="J28" s="52"/>
+      <c r="K28" s="52"/>
+      <c r="M28" s="53"/>
+    </row>
+    <row r="29" spans="1:13" ht="19.350000000000001" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A29" s="47">
         <f t="shared" si="3"/>
         <v>16</v>
       </c>
-      <c r="B29" s="12" t="str">
+      <c r="B29" s="48" t="str">
         <f t="shared" ref="B29:B39" si="4">IF(A29="","",CHOOSE(WEEKDAY(A29),"日","月","火","水","木","金","土"))</f>
         <v>月</v>
       </c>
-      <c r="C29" s="11"/>
-      <c r="D29" s="20"/>
-      <c r="E29" s="20"/>
-      <c r="F29" s="20"/>
-      <c r="G29" s="17"/>
-      <c r="H29" s="9"/>
-      <c r="I29" s="9"/>
-      <c r="J29" s="10"/>
-      <c r="K29" s="10"/>
-      <c r="M29" s="7"/>
-    </row>
-    <row r="30" spans="1:13" ht="19.350000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A30" s="8">
+      <c r="C29" s="49"/>
+      <c r="D29" s="50"/>
+      <c r="E29" s="50"/>
+      <c r="F29" s="50"/>
+      <c r="G29" s="63"/>
+      <c r="H29" s="51"/>
+      <c r="I29" s="51"/>
+      <c r="J29" s="52"/>
+      <c r="K29" s="52"/>
+      <c r="M29" s="53"/>
+    </row>
+    <row r="30" spans="1:13" ht="19.350000000000001" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A30" s="47">
         <f t="shared" si="3"/>
         <v>17</v>
       </c>
-      <c r="B30" s="12" t="str">
+      <c r="B30" s="48" t="str">
         <f t="shared" si="4"/>
         <v>火</v>
       </c>
-      <c r="C30" s="11"/>
-      <c r="D30" s="20"/>
-      <c r="E30" s="20"/>
-      <c r="F30" s="20"/>
-      <c r="G30" s="17"/>
-      <c r="H30" s="9"/>
-      <c r="I30" s="9"/>
-      <c r="J30" s="10"/>
-      <c r="K30" s="10"/>
-      <c r="M30" s="7"/>
-    </row>
-    <row r="31" spans="1:13" ht="19.350000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A31" s="8">
+      <c r="C30" s="49"/>
+      <c r="D30" s="50"/>
+      <c r="E30" s="50"/>
+      <c r="F30" s="50"/>
+      <c r="G30" s="63"/>
+      <c r="H30" s="51"/>
+      <c r="I30" s="51"/>
+      <c r="J30" s="52"/>
+      <c r="K30" s="52"/>
+      <c r="M30" s="53"/>
+    </row>
+    <row r="31" spans="1:13" ht="19.350000000000001" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A31" s="47">
         <f t="shared" si="3"/>
         <v>18</v>
       </c>
-      <c r="B31" s="12" t="str">
+      <c r="B31" s="48" t="str">
         <f t="shared" si="4"/>
         <v>水</v>
       </c>
-      <c r="C31" s="11"/>
-      <c r="D31" s="20"/>
-      <c r="E31" s="20"/>
-      <c r="F31" s="20"/>
-      <c r="G31" s="17"/>
-      <c r="H31" s="9"/>
-      <c r="I31" s="9"/>
-      <c r="J31" s="10"/>
-      <c r="K31" s="10"/>
-      <c r="M31" s="7"/>
-    </row>
-    <row r="32" spans="1:13" ht="19.350000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A32" s="8">
+      <c r="C31" s="49"/>
+      <c r="D31" s="50"/>
+      <c r="E31" s="50"/>
+      <c r="F31" s="50"/>
+      <c r="G31" s="63"/>
+      <c r="H31" s="51"/>
+      <c r="I31" s="51"/>
+      <c r="J31" s="52"/>
+      <c r="K31" s="52"/>
+      <c r="M31" s="53"/>
+    </row>
+    <row r="32" spans="1:13" ht="19.350000000000001" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A32" s="47">
         <f>A31+1</f>
         <v>19</v>
       </c>
-      <c r="B32" s="12" t="str">
+      <c r="B32" s="48" t="str">
         <f t="shared" si="4"/>
         <v>木</v>
       </c>
-      <c r="C32" s="11"/>
-      <c r="D32" s="20"/>
-      <c r="E32" s="20"/>
-      <c r="F32" s="20"/>
-      <c r="G32" s="17"/>
-      <c r="H32" s="9"/>
-      <c r="I32" s="9"/>
-      <c r="J32" s="10"/>
-      <c r="K32" s="10"/>
-      <c r="M32" s="7"/>
-    </row>
-    <row r="33" spans="1:13" ht="19.350000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A33" s="8">
+      <c r="C32" s="49"/>
+      <c r="D32" s="50"/>
+      <c r="E32" s="50"/>
+      <c r="F32" s="50"/>
+      <c r="G32" s="63"/>
+      <c r="H32" s="51"/>
+      <c r="I32" s="51"/>
+      <c r="J32" s="52"/>
+      <c r="K32" s="52"/>
+      <c r="M32" s="53"/>
+    </row>
+    <row r="33" spans="1:13" ht="19.350000000000001" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A33" s="47">
         <f>A32+1</f>
         <v>20</v>
       </c>
-      <c r="B33" s="12" t="str">
+      <c r="B33" s="48" t="str">
         <f t="shared" si="4"/>
         <v>金</v>
       </c>
-      <c r="C33" s="11"/>
-      <c r="D33" s="20"/>
-      <c r="E33" s="20"/>
-      <c r="F33" s="20"/>
-      <c r="G33" s="17"/>
-      <c r="H33" s="9"/>
-      <c r="I33" s="9"/>
-      <c r="J33" s="10"/>
-      <c r="K33" s="10"/>
-      <c r="M33" s="7"/>
-    </row>
-    <row r="34" spans="1:13" ht="19.350000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A34" s="8">
+      <c r="C33" s="49"/>
+      <c r="D33" s="50"/>
+      <c r="E33" s="50"/>
+      <c r="F33" s="50"/>
+      <c r="G33" s="63"/>
+      <c r="H33" s="51"/>
+      <c r="I33" s="51"/>
+      <c r="J33" s="52"/>
+      <c r="K33" s="52"/>
+      <c r="M33" s="53"/>
+    </row>
+    <row r="34" spans="1:13" ht="19.350000000000001" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A34" s="47">
         <f t="shared" ref="A34:A35" si="5">A33+1</f>
         <v>21</v>
       </c>
-      <c r="B34" s="12" t="str">
+      <c r="B34" s="48" t="str">
         <f t="shared" si="4"/>
         <v>土</v>
       </c>
-      <c r="C34" s="11"/>
-      <c r="D34" s="20"/>
-      <c r="E34" s="20"/>
-      <c r="F34" s="20"/>
-      <c r="G34" s="17"/>
-      <c r="H34" s="9"/>
-      <c r="I34" s="9"/>
-      <c r="J34" s="10"/>
-      <c r="K34" s="10"/>
-      <c r="M34" s="7"/>
-    </row>
-    <row r="35" spans="1:13" ht="19.350000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A35" s="8">
+      <c r="C34" s="49"/>
+      <c r="D34" s="50"/>
+      <c r="E34" s="50"/>
+      <c r="F34" s="50"/>
+      <c r="G34" s="63"/>
+      <c r="H34" s="51"/>
+      <c r="I34" s="51"/>
+      <c r="J34" s="52"/>
+      <c r="K34" s="52"/>
+      <c r="M34" s="53"/>
+    </row>
+    <row r="35" spans="1:13" ht="19.350000000000001" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A35" s="47">
         <f t="shared" si="5"/>
         <v>22</v>
       </c>
-      <c r="B35" s="12" t="str">
+      <c r="B35" s="48" t="str">
         <f t="shared" si="4"/>
         <v>日</v>
       </c>
-      <c r="C35" s="11"/>
-      <c r="D35" s="20"/>
-      <c r="E35" s="20"/>
-      <c r="F35" s="20"/>
-      <c r="G35" s="17"/>
-      <c r="H35" s="9"/>
-      <c r="I35" s="9"/>
-      <c r="J35" s="10"/>
-      <c r="K35" s="10"/>
-      <c r="M35" s="7"/>
-    </row>
-    <row r="36" spans="1:13" ht="19.350000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A36" s="8">
+      <c r="C35" s="49"/>
+      <c r="D35" s="50"/>
+      <c r="E35" s="50"/>
+      <c r="F35" s="50"/>
+      <c r="G35" s="63"/>
+      <c r="H35" s="51"/>
+      <c r="I35" s="51"/>
+      <c r="J35" s="52"/>
+      <c r="K35" s="52"/>
+      <c r="M35" s="53"/>
+    </row>
+    <row r="36" spans="1:13" ht="19.350000000000001" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A36" s="47">
         <f>A35+1</f>
         <v>23</v>
       </c>
-      <c r="B36" s="12" t="str">
+      <c r="B36" s="48" t="str">
         <f t="shared" si="4"/>
         <v>月</v>
       </c>
-      <c r="C36" s="11"/>
-      <c r="D36" s="20"/>
-      <c r="E36" s="20"/>
-      <c r="F36" s="20"/>
-      <c r="G36" s="17"/>
-      <c r="H36" s="9"/>
-      <c r="I36" s="9"/>
-      <c r="J36" s="10"/>
-      <c r="K36" s="10"/>
-      <c r="M36" s="7"/>
-    </row>
-    <row r="37" spans="1:13" ht="19.350000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A37" s="8">
+      <c r="C36" s="49"/>
+      <c r="D36" s="50"/>
+      <c r="E36" s="50"/>
+      <c r="F36" s="50"/>
+      <c r="G36" s="63"/>
+      <c r="H36" s="51"/>
+      <c r="I36" s="51"/>
+      <c r="J36" s="52"/>
+      <c r="K36" s="52"/>
+      <c r="M36" s="53"/>
+    </row>
+    <row r="37" spans="1:13" ht="19.350000000000001" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A37" s="47">
         <f>A36+1</f>
         <v>24</v>
       </c>
-      <c r="B37" s="12" t="str">
+      <c r="B37" s="48" t="str">
         <f t="shared" si="4"/>
         <v>火</v>
       </c>
-      <c r="C37" s="11"/>
-      <c r="D37" s="20"/>
-      <c r="E37" s="20"/>
-      <c r="F37" s="20"/>
-      <c r="G37" s="17"/>
-      <c r="H37" s="9"/>
-      <c r="I37" s="9"/>
-      <c r="J37" s="10"/>
-      <c r="K37" s="10"/>
-      <c r="M37" s="7"/>
-    </row>
-    <row r="38" spans="1:13" ht="19.350000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A38" s="8">
+      <c r="C37" s="49"/>
+      <c r="D37" s="50"/>
+      <c r="E37" s="50"/>
+      <c r="F37" s="50"/>
+      <c r="G37" s="63"/>
+      <c r="H37" s="51"/>
+      <c r="I37" s="51"/>
+      <c r="J37" s="52"/>
+      <c r="K37" s="52"/>
+      <c r="M37" s="53"/>
+    </row>
+    <row r="38" spans="1:13" ht="19.350000000000001" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A38" s="47">
         <f>A37+1</f>
         <v>25</v>
       </c>
-      <c r="B38" s="12" t="str">
+      <c r="B38" s="48" t="str">
         <f t="shared" si="4"/>
         <v>水</v>
       </c>
-      <c r="C38" s="11"/>
-      <c r="D38" s="20"/>
-      <c r="E38" s="20"/>
-      <c r="F38" s="20"/>
-      <c r="G38" s="17"/>
-      <c r="H38" s="9"/>
-      <c r="I38" s="9"/>
-      <c r="J38" s="10"/>
-      <c r="K38" s="10"/>
-      <c r="M38" s="7"/>
-    </row>
-    <row r="39" spans="1:13" ht="19.350000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A39" s="8">
+      <c r="C38" s="49"/>
+      <c r="D38" s="50"/>
+      <c r="E38" s="50"/>
+      <c r="F38" s="50"/>
+      <c r="G38" s="63"/>
+      <c r="H38" s="51"/>
+      <c r="I38" s="51"/>
+      <c r="J38" s="52"/>
+      <c r="K38" s="52"/>
+      <c r="M38" s="53"/>
+    </row>
+    <row r="39" spans="1:13" ht="19.350000000000001" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A39" s="47">
         <f>A38+1</f>
         <v>26</v>
       </c>
-      <c r="B39" s="12" t="str">
+      <c r="B39" s="48" t="str">
         <f t="shared" si="4"/>
         <v>木</v>
       </c>
-      <c r="C39" s="11"/>
-      <c r="D39" s="20"/>
-      <c r="E39" s="20"/>
-      <c r="F39" s="20"/>
-      <c r="G39" s="17"/>
-      <c r="H39" s="9"/>
-      <c r="I39" s="9"/>
-      <c r="J39" s="10"/>
-      <c r="K39" s="10"/>
-      <c r="M39" s="7"/>
-    </row>
-    <row r="40" spans="1:13" ht="19.350000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A40" s="8">
+      <c r="C39" s="49"/>
+      <c r="D39" s="50"/>
+      <c r="E39" s="50"/>
+      <c r="F39" s="50"/>
+      <c r="G39" s="63"/>
+      <c r="H39" s="51"/>
+      <c r="I39" s="51"/>
+      <c r="J39" s="52"/>
+      <c r="K39" s="52"/>
+      <c r="M39" s="53"/>
+    </row>
+    <row r="40" spans="1:13" ht="19.350000000000001" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A40" s="47">
         <f t="shared" ref="A40:A41" si="6">A39+1</f>
         <v>27</v>
       </c>
-      <c r="B40" s="12" t="str">
+      <c r="B40" s="48" t="str">
         <f t="shared" ref="B40:B43" si="7">IF(A40="","",CHOOSE(WEEKDAY(A40),"日","月","火","水","木","金","土"))</f>
         <v>金</v>
       </c>
-      <c r="C40" s="11"/>
-      <c r="D40" s="20"/>
-      <c r="E40" s="20"/>
-      <c r="F40" s="20"/>
-      <c r="G40" s="17"/>
-      <c r="H40" s="9"/>
-      <c r="I40" s="9"/>
-      <c r="J40" s="10"/>
-      <c r="K40" s="10"/>
-      <c r="M40" s="7"/>
-    </row>
-    <row r="41" spans="1:13" ht="19.350000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A41" s="8">
+      <c r="C40" s="49"/>
+      <c r="D40" s="50"/>
+      <c r="E40" s="50"/>
+      <c r="F40" s="50"/>
+      <c r="G40" s="63"/>
+      <c r="H40" s="51"/>
+      <c r="I40" s="51"/>
+      <c r="J40" s="52"/>
+      <c r="K40" s="52"/>
+      <c r="M40" s="53"/>
+    </row>
+    <row r="41" spans="1:13" ht="19.350000000000001" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A41" s="47">
         <f t="shared" si="6"/>
         <v>28</v>
       </c>
-      <c r="B41" s="12" t="str">
+      <c r="B41" s="48" t="str">
         <f t="shared" si="7"/>
         <v>土</v>
       </c>
-      <c r="C41" s="11"/>
-      <c r="D41" s="20"/>
-      <c r="E41" s="20"/>
-      <c r="F41" s="20"/>
-      <c r="G41" s="17"/>
-      <c r="H41" s="9"/>
-      <c r="I41" s="9"/>
-      <c r="J41" s="10"/>
-      <c r="K41" s="10"/>
-      <c r="M41" s="7"/>
-    </row>
-    <row r="42" spans="1:13" ht="19.350000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A42" s="8">
+      <c r="C41" s="49"/>
+      <c r="D41" s="50"/>
+      <c r="E41" s="50"/>
+      <c r="F41" s="50"/>
+      <c r="G41" s="63"/>
+      <c r="H41" s="51"/>
+      <c r="I41" s="51"/>
+      <c r="J41" s="52"/>
+      <c r="K41" s="52"/>
+      <c r="M41" s="53"/>
+    </row>
+    <row r="42" spans="1:13" ht="19.350000000000001" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A42" s="47">
         <f>A41+1</f>
         <v>29</v>
       </c>
-      <c r="B42" s="12" t="str">
+      <c r="B42" s="48" t="str">
         <f t="shared" si="7"/>
         <v>日</v>
       </c>
-      <c r="C42" s="11"/>
-      <c r="D42" s="20"/>
-      <c r="E42" s="20"/>
-      <c r="F42" s="20"/>
-      <c r="G42" s="28"/>
-      <c r="H42" s="9"/>
-      <c r="I42" s="9"/>
-      <c r="J42" s="10"/>
-      <c r="K42" s="10"/>
-      <c r="M42" s="7"/>
-    </row>
-    <row r="43" spans="1:13" ht="19.350000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A43" s="8">
+      <c r="C42" s="49"/>
+      <c r="D42" s="50"/>
+      <c r="E42" s="50"/>
+      <c r="F42" s="50"/>
+      <c r="G42" s="64"/>
+      <c r="H42" s="51"/>
+      <c r="I42" s="51"/>
+      <c r="J42" s="52"/>
+      <c r="K42" s="52"/>
+      <c r="M42" s="53"/>
+    </row>
+    <row r="43" spans="1:13" ht="19.350000000000001" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A43" s="47">
         <f>A42+1</f>
         <v>30</v>
       </c>
-      <c r="B43" s="12" t="str">
+      <c r="B43" s="48" t="str">
         <f t="shared" si="7"/>
         <v>月</v>
       </c>
-      <c r="C43" s="11"/>
-      <c r="D43" s="20"/>
-      <c r="E43" s="20"/>
-      <c r="F43" s="20"/>
-      <c r="G43" s="28"/>
-      <c r="H43" s="9"/>
-      <c r="I43" s="9"/>
-      <c r="J43" s="10"/>
-      <c r="K43" s="10"/>
-      <c r="M43" s="7"/>
-    </row>
-    <row r="44" spans="1:13" ht="19.350000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A44" s="29" t="s">
+      <c r="C43" s="49"/>
+      <c r="D43" s="50"/>
+      <c r="E43" s="50"/>
+      <c r="F43" s="50"/>
+      <c r="G43" s="64"/>
+      <c r="H43" s="51"/>
+      <c r="I43" s="51"/>
+      <c r="J43" s="52"/>
+      <c r="K43" s="52"/>
+      <c r="M43" s="53"/>
+    </row>
+    <row r="44" spans="1:13" ht="19.350000000000001" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A44" s="54" t="s">
         <v>23</v>
       </c>
-      <c r="B44" s="30"/>
-      <c r="C44" s="18">
+      <c r="B44" s="55"/>
+      <c r="C44" s="56">
         <f>COUNTA(H13:H43)</f>
         <v>0</v>
       </c>
-      <c r="D44" s="13" t="s">
+      <c r="D44" s="57" t="s">
         <v>15</v>
       </c>
-      <c r="E44" s="19" t="s">
+      <c r="E44" s="58" t="s">
         <v>22</v>
       </c>
-      <c r="F44" s="27">
+      <c r="F44" s="59">
         <f>(SUM(K13:K43)/TIME(1,,))</f>
         <v>0</v>
       </c>
-      <c r="G44" s="13" t="s">
+      <c r="G44" s="57" t="s">
         <v>24</v>
       </c>
-      <c r="H44" s="19" t="s">
+      <c r="H44" s="58" t="s">
         <v>25</v>
       </c>
-      <c r="I44" s="14">
+      <c r="I44" s="60">
         <f>$F$44-$C$44*8</f>
         <v>0</v>
       </c>
-      <c r="J44" s="15" t="s">
+      <c r="J44" s="61" t="s">
         <v>24</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="20">
-    <mergeCell ref="A2:H2"/>
-    <mergeCell ref="I2:K2"/>
-    <mergeCell ref="A3:C3"/>
-    <mergeCell ref="D3:H3"/>
-    <mergeCell ref="A4:C4"/>
-    <mergeCell ref="D4:H4"/>
     <mergeCell ref="A44:B44"/>
     <mergeCell ref="A5:C5"/>
     <mergeCell ref="D5:H5"/>
@@ -1850,11 +1844,17 @@
     <mergeCell ref="G9:H9"/>
     <mergeCell ref="A10:C10"/>
     <mergeCell ref="D10:H10"/>
+    <mergeCell ref="A2:H2"/>
+    <mergeCell ref="I2:K2"/>
+    <mergeCell ref="A3:C3"/>
+    <mergeCell ref="D3:H3"/>
+    <mergeCell ref="A4:C4"/>
+    <mergeCell ref="D4:H4"/>
   </mergeCells>
-  <phoneticPr fontId="9"/>
+  <phoneticPr fontId="3"/>
   <printOptions horizontalCentered="1"/>
   <pageMargins left="0.78740157480314965" right="0.78740157480314965" top="0.78740157480314965" bottom="0.19685039370078741" header="0.51181102362204722" footer="0.11811023622047245"/>
-  <pageSetup paperSize="9" scale="92" orientation="portrait" horizontalDpi="300" verticalDpi="300" r:id="rId1"/>
+  <pageSetup paperSize="9" scale="93" orientation="portrait" horizontalDpi="300" verticalDpi="300" r:id="rId1"/>
   <headerFooter alignWithMargins="0">
     <oddHeader>&amp;R&amp;"Arial,太字"&amp;12&amp;K00-049Highly Confidential</oddHeader>
   </headerFooter>
@@ -1862,6 +1862,26 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="fddd5c7a-2dc9-4280-9104-0c5c090f8913">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <TaxCatchAll xmlns="49da8719-5195-4d58-b9e3-040d669e384e" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100DC957A2BAE3FEB488DD90F3CEEBA64B2" ma:contentTypeVersion="12" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="5f1653939578ce63f276984d74f7b80f">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="fddd5c7a-2dc9-4280-9104-0c5c090f8913" xmlns:ns3="49da8719-5195-4d58-b9e3-040d669e384e" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="31f706c199e200b5ceeaeb3f8c022435" ns2:_="" ns3:_="">
     <xsd:import namespace="fddd5c7a-2dc9-4280-9104-0c5c090f8913"/>
@@ -2062,27 +2082,27 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{A7A8AE5A-FCD2-4F3B-B711-AC3CFBE815ED}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="43eb3a32-fd45-4fa4-b7b4-e786cec62659"/>
+    <ds:schemaRef ds:uri="fddd5c7a-2dc9-4280-9104-0c5c090f8913"/>
+    <ds:schemaRef ds:uri="49da8719-5195-4d58-b9e3-040d669e384e"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="fddd5c7a-2dc9-4280-9104-0c5c090f8913">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-    <TaxCatchAll xmlns="49da8719-5195-4d58-b9e3-040d669e384e" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{F9C41F5C-CAF1-47CB-985C-96AFA693AEFA}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{27D2DB86-FB68-473C-AC36-38170BDA1492}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -2099,24 +2119,4 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{F9C41F5C-CAF1-47CB-985C-96AFA693AEFA}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{A7A8AE5A-FCD2-4F3B-B711-AC3CFBE815ED}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="43eb3a32-fd45-4fa4-b7b4-e786cec62659"/>
-    <ds:schemaRef ds:uri="fddd5c7a-2dc9-4280-9104-0c5c090f8913"/>
-    <ds:schemaRef ds:uri="49da8719-5195-4d58-b9e3-040d669e384e"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
 </file>
</xml_diff>

<commit_message>
Add fixed-time mode and additional breaks feature with proper validation and formatting
</commit_message>
<xml_diff>
--- a/templates/Excel_templates/タイムシート(yyyy_mm).xlsx
+++ b/templates/Excel_templates/タイムシート(yyyy_mm).xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\kenichi.yamamoto\Documents\wk_src\timesheet-api\templates\Excel_templates\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7E086512-C782-410F-B9B1-6C9336D733E2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{935B9F14-0B47-4066-96C3-B095CCFA595E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -514,6 +514,114 @@
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="2" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="8" fillId="0" borderId="10" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="14" fontId="8" fillId="0" borderId="10" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="6" fillId="2" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="centerContinuous" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="centerContinuous" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="2" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="centerContinuous" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="2" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="centerContinuous" vertical="center" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="12" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="centerContinuous" vertical="center"/>
+    </xf>
+    <xf numFmtId="176" fontId="6" fillId="0" borderId="9" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="9" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="centerContinuous" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="9" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="2" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="20" fontId="10" fillId="0" borderId="9" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="20" fontId="10" fillId="0" borderId="13" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="20" fontId="6" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="38" fontId="10" fillId="0" borderId="1" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="2" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="20" fontId="10" fillId="0" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="10" fillId="0" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="3" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="6" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="3" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="2" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="6" fillId="0" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="6" fillId="0" borderId="3" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="3" borderId="4" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="3" borderId="0" xfId="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="3" borderId="8" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="1" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="2" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="3" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="3" borderId="9" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="3" borderId="10" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="3" borderId="11" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="49" fontId="7" fillId="3" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
@@ -523,6 +631,48 @@
     <xf numFmtId="49" fontId="7" fillId="3" borderId="3" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
+    <xf numFmtId="49" fontId="8" fillId="3" borderId="5" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="8" fillId="3" borderId="6" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="8" fillId="3" borderId="7" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="4" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="8" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="1" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="2" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="3" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="8" fillId="3" borderId="4" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="8" fillId="3" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="8" fillId="3" borderId="8" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="14" fontId="8" fillId="4" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="14" fontId="8" fillId="4" borderId="2" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="14" fontId="8" fillId="4" borderId="3" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="14" fontId="6" fillId="0" borderId="4" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
     </xf>
@@ -546,156 +696,6 @@
     </xf>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="3" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="3" borderId="4" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="3" borderId="0" xfId="1" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="3" borderId="8" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="1" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="2" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="3" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="3" borderId="9" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="3" borderId="10" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="3" borderId="11" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="8" fillId="3" borderId="5" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="8" fillId="3" borderId="6" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="8" fillId="3" borderId="7" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="4" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="8" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="1" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="2" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="3" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="8" fillId="3" borderId="4" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="8" fillId="3" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="8" fillId="3" borderId="8" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="14" fontId="8" fillId="4" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="14" fontId="8" fillId="4" borderId="2" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="2" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="14" fontId="8" fillId="4" borderId="3" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="8" fillId="0" borderId="10" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="14" fontId="8" fillId="0" borderId="10" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="6" fillId="2" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="centerContinuous" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="2" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="centerContinuous" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="2" borderId="2" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="centerContinuous" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="2" borderId="2" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="centerContinuous" vertical="center" shrinkToFit="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="2" borderId="12" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="centerContinuous" vertical="center"/>
-    </xf>
-    <xf numFmtId="176" fontId="6" fillId="0" borderId="9" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="9" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="centerContinuous" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="9" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="2" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="20" fontId="10" fillId="0" borderId="9" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="20" fontId="10" fillId="0" borderId="13" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="20" fontId="6" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="6" fillId="0" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="6" fillId="0" borderId="3" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="38" fontId="10" fillId="0" borderId="1" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="2" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="20" fontId="10" fillId="0" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="2" fontId="10" fillId="0" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="3" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="6" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="3" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="2" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="3">
@@ -985,7 +985,7 @@
   <dimension ref="A1:M44"/>
   <sheetFormatPr defaultColWidth="7.26953125" defaultRowHeight="15" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="3.08984375" style="62" customWidth="1"/>
+    <col min="1" max="1" width="3.08984375" style="26" customWidth="1"/>
     <col min="2" max="2" width="3.08984375" style="3" customWidth="1"/>
     <col min="3" max="3" width="7.453125" style="3" customWidth="1"/>
     <col min="4" max="7" width="8.08984375" style="3" customWidth="1"/>
@@ -1012,824 +1012,830 @@
       <c r="K1" s="2"/>
     </row>
     <row r="2" spans="1:13" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A2" s="4" t="s">
+      <c r="A2" s="40" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="5"/>
-      <c r="C2" s="5"/>
-      <c r="D2" s="5"/>
-      <c r="E2" s="5"/>
-      <c r="F2" s="5"/>
-      <c r="G2" s="5"/>
-      <c r="H2" s="6"/>
-      <c r="I2" s="7">
+      <c r="B2" s="41"/>
+      <c r="C2" s="41"/>
+      <c r="D2" s="41"/>
+      <c r="E2" s="41"/>
+      <c r="F2" s="41"/>
+      <c r="G2" s="41"/>
+      <c r="H2" s="42"/>
+      <c r="I2" s="57">
         <f>G9+1</f>
         <v>1</v>
       </c>
-      <c r="J2" s="8"/>
-      <c r="K2" s="8"/>
+      <c r="J2" s="58"/>
+      <c r="K2" s="58"/>
     </row>
     <row r="3" spans="1:13" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A3" s="9" t="s">
+      <c r="A3" s="59" t="s">
         <v>2</v>
       </c>
-      <c r="B3" s="10"/>
-      <c r="C3" s="11"/>
-      <c r="D3" s="12" t="s">
+      <c r="B3" s="60"/>
+      <c r="C3" s="61"/>
+      <c r="D3" s="62" t="s">
         <v>3</v>
       </c>
-      <c r="E3" s="13"/>
-      <c r="F3" s="13"/>
-      <c r="G3" s="13"/>
-      <c r="H3" s="14"/>
+      <c r="E3" s="63"/>
+      <c r="F3" s="63"/>
+      <c r="G3" s="63"/>
+      <c r="H3" s="64"/>
     </row>
     <row r="4" spans="1:13" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A4" s="15" t="s">
+      <c r="A4" s="31" t="s">
         <v>4</v>
       </c>
-      <c r="B4" s="16"/>
-      <c r="C4" s="17"/>
-      <c r="D4" s="18" t="s">
+      <c r="B4" s="32"/>
+      <c r="C4" s="33"/>
+      <c r="D4" s="34" t="s">
         <v>26</v>
       </c>
-      <c r="E4" s="19"/>
-      <c r="F4" s="19"/>
-      <c r="G4" s="19"/>
-      <c r="H4" s="20"/>
+      <c r="E4" s="35"/>
+      <c r="F4" s="35"/>
+      <c r="G4" s="35"/>
+      <c r="H4" s="36"/>
     </row>
     <row r="5" spans="1:13" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A5" s="15" t="s">
+      <c r="A5" s="31" t="s">
         <v>5</v>
       </c>
-      <c r="B5" s="16"/>
-      <c r="C5" s="17"/>
-      <c r="D5" s="18" t="s">
+      <c r="B5" s="32"/>
+      <c r="C5" s="33"/>
+      <c r="D5" s="34" t="s">
         <v>6</v>
       </c>
-      <c r="E5" s="19"/>
-      <c r="F5" s="19"/>
-      <c r="G5" s="19"/>
-      <c r="H5" s="20"/>
+      <c r="E5" s="35"/>
+      <c r="F5" s="35"/>
+      <c r="G5" s="35"/>
+      <c r="H5" s="36"/>
     </row>
     <row r="6" spans="1:13" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A6" s="21" t="s">
+      <c r="A6" s="37" t="s">
         <v>7</v>
       </c>
-      <c r="B6" s="22"/>
-      <c r="C6" s="23"/>
-      <c r="D6" s="18"/>
-      <c r="E6" s="19"/>
-      <c r="F6" s="19"/>
-      <c r="G6" s="19"/>
-      <c r="H6" s="20"/>
+      <c r="B6" s="38"/>
+      <c r="C6" s="39"/>
+      <c r="D6" s="34"/>
+      <c r="E6" s="35"/>
+      <c r="F6" s="35"/>
+      <c r="G6" s="35"/>
+      <c r="H6" s="36"/>
     </row>
     <row r="7" spans="1:13" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A7" s="4" t="s">
+      <c r="A7" s="40" t="s">
         <v>8</v>
       </c>
-      <c r="B7" s="5"/>
-      <c r="C7" s="5"/>
-      <c r="D7" s="5"/>
-      <c r="E7" s="5"/>
-      <c r="F7" s="5"/>
-      <c r="G7" s="5"/>
-      <c r="H7" s="6"/>
+      <c r="B7" s="41"/>
+      <c r="C7" s="41"/>
+      <c r="D7" s="41"/>
+      <c r="E7" s="41"/>
+      <c r="F7" s="41"/>
+      <c r="G7" s="41"/>
+      <c r="H7" s="42"/>
     </row>
     <row r="8" spans="1:13" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A8" s="24" t="s">
+      <c r="A8" s="43" t="s">
         <v>9</v>
       </c>
-      <c r="B8" s="25"/>
-      <c r="C8" s="26"/>
-      <c r="D8" s="27"/>
-      <c r="E8" s="28"/>
-      <c r="F8" s="29" t="s">
+      <c r="B8" s="44"/>
+      <c r="C8" s="45"/>
+      <c r="D8" s="46"/>
+      <c r="E8" s="47"/>
+      <c r="F8" s="48" t="s">
         <v>10</v>
       </c>
-      <c r="G8" s="30"/>
-      <c r="H8" s="31"/>
+      <c r="G8" s="49"/>
+      <c r="H8" s="50"/>
     </row>
     <row r="9" spans="1:13" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A9" s="32" t="s">
+      <c r="A9" s="51" t="s">
         <v>11</v>
       </c>
-      <c r="B9" s="33"/>
-      <c r="C9" s="34"/>
-      <c r="D9" s="35"/>
-      <c r="E9" s="36"/>
-      <c r="F9" s="37" t="s">
+      <c r="B9" s="52"/>
+      <c r="C9" s="53"/>
+      <c r="D9" s="54"/>
+      <c r="E9" s="55"/>
+      <c r="F9" s="4" t="s">
         <v>12</v>
       </c>
-      <c r="G9" s="36"/>
-      <c r="H9" s="38"/>
+      <c r="G9" s="55"/>
+      <c r="H9" s="56"/>
     </row>
     <row r="10" spans="1:13" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A10" s="21" t="s">
+      <c r="A10" s="37" t="s">
         <v>13</v>
       </c>
-      <c r="B10" s="22"/>
-      <c r="C10" s="23"/>
-      <c r="D10" s="18" t="s">
+      <c r="B10" s="38"/>
+      <c r="C10" s="39"/>
+      <c r="D10" s="34" t="s">
         <v>14</v>
       </c>
-      <c r="E10" s="19"/>
-      <c r="F10" s="19"/>
-      <c r="G10" s="19"/>
-      <c r="H10" s="20"/>
+      <c r="E10" s="35"/>
+      <c r="F10" s="35"/>
+      <c r="G10" s="35"/>
+      <c r="H10" s="36"/>
     </row>
     <row r="11" spans="1:13" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A11" s="39"/>
-      <c r="B11" s="39"/>
-      <c r="C11" s="40"/>
-      <c r="D11" s="40"/>
-      <c r="E11" s="41"/>
-      <c r="F11" s="40"/>
-      <c r="G11" s="40"/>
+      <c r="A11" s="5"/>
+      <c r="B11" s="5"/>
+      <c r="C11" s="6"/>
+      <c r="D11" s="6"/>
+      <c r="E11" s="7"/>
+      <c r="F11" s="6"/>
+      <c r="G11" s="6"/>
     </row>
     <row r="12" spans="1:13" ht="19.350000000000001" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A12" s="42" t="s">
+      <c r="A12" s="8" t="s">
         <v>15</v>
       </c>
-      <c r="B12" s="43" t="s">
+      <c r="B12" s="9" t="s">
         <v>16</v>
       </c>
-      <c r="C12" s="43" t="s">
+      <c r="C12" s="9" t="s">
         <v>17</v>
       </c>
-      <c r="D12" s="44"/>
-      <c r="E12" s="44"/>
-      <c r="F12" s="44"/>
-      <c r="G12" s="45" t="s">
+      <c r="D12" s="10"/>
+      <c r="E12" s="10"/>
+      <c r="F12" s="10"/>
+      <c r="G12" s="11" t="s">
         <v>18</v>
       </c>
-      <c r="H12" s="43" t="s">
+      <c r="H12" s="9" t="s">
         <v>19</v>
       </c>
-      <c r="I12" s="43" t="s">
+      <c r="I12" s="9" t="s">
         <v>20</v>
       </c>
-      <c r="J12" s="46" t="s">
+      <c r="J12" s="12" t="s">
         <v>21</v>
       </c>
-      <c r="K12" s="46" t="s">
+      <c r="K12" s="12" t="s">
         <v>22</v>
       </c>
     </row>
     <row r="13" spans="1:13" ht="19.350000000000001" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A13" s="47">
+      <c r="A13" s="13">
         <f>D9</f>
         <v>0</v>
       </c>
-      <c r="B13" s="48" t="str">
+      <c r="B13" s="14" t="str">
         <f>IF(A13="","",CHOOSE(WEEKDAY(A13),"日","月","火","水","木","金","土"))</f>
         <v>土</v>
       </c>
-      <c r="C13" s="49"/>
-      <c r="D13" s="50"/>
-      <c r="E13" s="50"/>
-      <c r="F13" s="50"/>
-      <c r="G13" s="63"/>
-      <c r="H13" s="51"/>
-      <c r="I13" s="51"/>
-      <c r="J13" s="52"/>
-      <c r="K13" s="52"/>
-      <c r="M13" s="53"/>
+      <c r="C13" s="15"/>
+      <c r="D13" s="16"/>
+      <c r="E13" s="16"/>
+      <c r="F13" s="16"/>
+      <c r="G13" s="27"/>
+      <c r="H13" s="17"/>
+      <c r="I13" s="17"/>
+      <c r="J13" s="18"/>
+      <c r="K13" s="18"/>
+      <c r="M13" s="19"/>
     </row>
     <row r="14" spans="1:13" ht="19.350000000000001" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A14" s="47">
+      <c r="A14" s="13">
         <f>A13+1</f>
         <v>1</v>
       </c>
-      <c r="B14" s="48" t="str">
+      <c r="B14" s="14" t="str">
         <f t="shared" ref="B14:B20" si="0">IF(A14="","",CHOOSE(WEEKDAY(A14),"日","月","火","水","木","金","土"))</f>
         <v>日</v>
       </c>
-      <c r="C14" s="49"/>
-      <c r="D14" s="50"/>
-      <c r="E14" s="50"/>
-      <c r="F14" s="50"/>
-      <c r="G14" s="63"/>
-      <c r="H14" s="51"/>
-      <c r="I14" s="51"/>
-      <c r="J14" s="52"/>
-      <c r="K14" s="52"/>
-      <c r="M14" s="53"/>
+      <c r="C14" s="15"/>
+      <c r="D14" s="16"/>
+      <c r="E14" s="16"/>
+      <c r="F14" s="16"/>
+      <c r="G14" s="27"/>
+      <c r="H14" s="17"/>
+      <c r="I14" s="17"/>
+      <c r="J14" s="18"/>
+      <c r="K14" s="18"/>
+      <c r="M14" s="19"/>
     </row>
     <row r="15" spans="1:13" ht="19.350000000000001" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A15" s="47">
+      <c r="A15" s="13">
         <f>A14+1</f>
         <v>2</v>
       </c>
-      <c r="B15" s="48" t="str">
+      <c r="B15" s="14" t="str">
         <f t="shared" si="0"/>
         <v>月</v>
       </c>
-      <c r="C15" s="49"/>
-      <c r="D15" s="50"/>
-      <c r="E15" s="50"/>
-      <c r="F15" s="50"/>
-      <c r="G15" s="63"/>
-      <c r="H15" s="51"/>
-      <c r="I15" s="51"/>
-      <c r="J15" s="52"/>
-      <c r="K15" s="52"/>
-      <c r="M15" s="53"/>
+      <c r="C15" s="15"/>
+      <c r="D15" s="16"/>
+      <c r="E15" s="16"/>
+      <c r="F15" s="16"/>
+      <c r="G15" s="27"/>
+      <c r="H15" s="17"/>
+      <c r="I15" s="17"/>
+      <c r="J15" s="18"/>
+      <c r="K15" s="18"/>
+      <c r="M15" s="19"/>
     </row>
     <row r="16" spans="1:13" ht="19.350000000000001" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A16" s="47">
+      <c r="A16" s="13">
         <f>A15+1</f>
         <v>3</v>
       </c>
-      <c r="B16" s="48" t="str">
+      <c r="B16" s="14" t="str">
         <f t="shared" si="0"/>
         <v>火</v>
       </c>
-      <c r="C16" s="49"/>
-      <c r="D16" s="50"/>
-      <c r="E16" s="50"/>
-      <c r="F16" s="50"/>
-      <c r="G16" s="63"/>
-      <c r="H16" s="51"/>
-      <c r="I16" s="51"/>
-      <c r="J16" s="52"/>
-      <c r="K16" s="52"/>
-      <c r="M16" s="53"/>
+      <c r="C16" s="15"/>
+      <c r="D16" s="16"/>
+      <c r="E16" s="16"/>
+      <c r="F16" s="16"/>
+      <c r="G16" s="27"/>
+      <c r="H16" s="17"/>
+      <c r="I16" s="17"/>
+      <c r="J16" s="18"/>
+      <c r="K16" s="18"/>
+      <c r="M16" s="19"/>
     </row>
     <row r="17" spans="1:13" ht="19.350000000000001" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A17" s="47">
+      <c r="A17" s="13">
         <f>A16+1</f>
         <v>4</v>
       </c>
-      <c r="B17" s="48" t="str">
+      <c r="B17" s="14" t="str">
         <f t="shared" si="0"/>
         <v>水</v>
       </c>
-      <c r="C17" s="49"/>
-      <c r="D17" s="50"/>
-      <c r="E17" s="50"/>
-      <c r="F17" s="50"/>
-      <c r="G17" s="63"/>
-      <c r="H17" s="51"/>
-      <c r="I17" s="51"/>
-      <c r="J17" s="52"/>
-      <c r="K17" s="52"/>
-      <c r="M17" s="53"/>
+      <c r="C17" s="15"/>
+      <c r="D17" s="16"/>
+      <c r="E17" s="16"/>
+      <c r="F17" s="16"/>
+      <c r="G17" s="27"/>
+      <c r="H17" s="17"/>
+      <c r="I17" s="17"/>
+      <c r="J17" s="18"/>
+      <c r="K17" s="18"/>
+      <c r="M17" s="19"/>
     </row>
     <row r="18" spans="1:13" ht="19.350000000000001" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A18" s="47">
+      <c r="A18" s="13">
         <f>A17+1</f>
         <v>5</v>
       </c>
-      <c r="B18" s="48" t="str">
+      <c r="B18" s="14" t="str">
         <f t="shared" si="0"/>
         <v>木</v>
       </c>
-      <c r="C18" s="49"/>
-      <c r="D18" s="50"/>
-      <c r="E18" s="50"/>
-      <c r="F18" s="50"/>
-      <c r="G18" s="63"/>
-      <c r="H18" s="51"/>
-      <c r="I18" s="51"/>
-      <c r="J18" s="52"/>
-      <c r="K18" s="52"/>
-      <c r="M18" s="53"/>
+      <c r="C18" s="15"/>
+      <c r="D18" s="16"/>
+      <c r="E18" s="16"/>
+      <c r="F18" s="16"/>
+      <c r="G18" s="27"/>
+      <c r="H18" s="17"/>
+      <c r="I18" s="17"/>
+      <c r="J18" s="18"/>
+      <c r="K18" s="18"/>
+      <c r="M18" s="19"/>
     </row>
     <row r="19" spans="1:13" ht="19.350000000000001" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A19" s="47">
+      <c r="A19" s="13">
         <f t="shared" ref="A19:A20" si="1">A18+1</f>
         <v>6</v>
       </c>
-      <c r="B19" s="48" t="str">
+      <c r="B19" s="14" t="str">
         <f t="shared" si="0"/>
         <v>金</v>
       </c>
-      <c r="C19" s="49"/>
-      <c r="D19" s="50"/>
-      <c r="E19" s="50"/>
-      <c r="F19" s="50"/>
-      <c r="G19" s="63"/>
-      <c r="H19" s="51"/>
-      <c r="I19" s="51"/>
-      <c r="J19" s="52"/>
-      <c r="K19" s="52"/>
-      <c r="M19" s="53"/>
+      <c r="C19" s="15"/>
+      <c r="D19" s="16"/>
+      <c r="E19" s="16"/>
+      <c r="F19" s="16"/>
+      <c r="G19" s="27"/>
+      <c r="H19" s="17"/>
+      <c r="I19" s="17"/>
+      <c r="J19" s="18"/>
+      <c r="K19" s="18"/>
+      <c r="M19" s="19"/>
     </row>
     <row r="20" spans="1:13" ht="19.350000000000001" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A20" s="47">
+      <c r="A20" s="13">
         <f t="shared" si="1"/>
         <v>7</v>
       </c>
-      <c r="B20" s="48" t="str">
+      <c r="B20" s="14" t="str">
         <f t="shared" si="0"/>
         <v>土</v>
       </c>
-      <c r="C20" s="49"/>
-      <c r="D20" s="50"/>
-      <c r="E20" s="50"/>
-      <c r="F20" s="50"/>
-      <c r="G20" s="63"/>
-      <c r="H20" s="51"/>
-      <c r="I20" s="51"/>
-      <c r="J20" s="52"/>
-      <c r="K20" s="52"/>
-      <c r="M20" s="53"/>
+      <c r="C20" s="15"/>
+      <c r="D20" s="16"/>
+      <c r="E20" s="16"/>
+      <c r="F20" s="16"/>
+      <c r="G20" s="27"/>
+      <c r="H20" s="17"/>
+      <c r="I20" s="17"/>
+      <c r="J20" s="18"/>
+      <c r="K20" s="18"/>
+      <c r="M20" s="19"/>
     </row>
     <row r="21" spans="1:13" ht="19.350000000000001" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A21" s="47">
+      <c r="A21" s="13">
         <f>A20+1</f>
         <v>8</v>
       </c>
-      <c r="B21" s="48" t="str">
+      <c r="B21" s="14" t="str">
         <f t="shared" ref="B21:B27" si="2">IF(A21="","",CHOOSE(WEEKDAY(A21),"日","月","火","水","木","金","土"))</f>
         <v>日</v>
       </c>
-      <c r="C21" s="49"/>
-      <c r="D21" s="50"/>
-      <c r="E21" s="50"/>
-      <c r="F21" s="50"/>
-      <c r="G21" s="63"/>
-      <c r="H21" s="51"/>
-      <c r="I21" s="51"/>
-      <c r="J21" s="52"/>
-      <c r="K21" s="52"/>
-      <c r="M21" s="53"/>
+      <c r="C21" s="15"/>
+      <c r="D21" s="16"/>
+      <c r="E21" s="16"/>
+      <c r="F21" s="16"/>
+      <c r="G21" s="27"/>
+      <c r="H21" s="17"/>
+      <c r="I21" s="17"/>
+      <c r="J21" s="18"/>
+      <c r="K21" s="18"/>
+      <c r="M21" s="19"/>
     </row>
     <row r="22" spans="1:13" ht="19.350000000000001" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A22" s="47">
+      <c r="A22" s="13">
         <f>A21+1</f>
         <v>9</v>
       </c>
-      <c r="B22" s="48" t="str">
+      <c r="B22" s="14" t="str">
         <f t="shared" si="2"/>
         <v>月</v>
       </c>
-      <c r="C22" s="49"/>
-      <c r="D22" s="50"/>
-      <c r="E22" s="50"/>
-      <c r="F22" s="50"/>
-      <c r="G22" s="63"/>
-      <c r="H22" s="51"/>
-      <c r="I22" s="51"/>
-      <c r="J22" s="52"/>
-      <c r="K22" s="52"/>
-      <c r="M22" s="53"/>
+      <c r="C22" s="15"/>
+      <c r="D22" s="16"/>
+      <c r="E22" s="16"/>
+      <c r="F22" s="16"/>
+      <c r="G22" s="27"/>
+      <c r="H22" s="17"/>
+      <c r="I22" s="17"/>
+      <c r="J22" s="18"/>
+      <c r="K22" s="18"/>
+      <c r="M22" s="19"/>
     </row>
     <row r="23" spans="1:13" ht="19.350000000000001" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A23" s="47">
+      <c r="A23" s="13">
         <f>A22+1</f>
         <v>10</v>
       </c>
-      <c r="B23" s="48" t="str">
+      <c r="B23" s="14" t="str">
         <f t="shared" si="2"/>
         <v>火</v>
       </c>
-      <c r="C23" s="49"/>
-      <c r="D23" s="50"/>
-      <c r="E23" s="50"/>
-      <c r="F23" s="50"/>
-      <c r="G23" s="63"/>
-      <c r="H23" s="51"/>
-      <c r="I23" s="51"/>
-      <c r="J23" s="52"/>
-      <c r="K23" s="52"/>
-      <c r="M23" s="53"/>
+      <c r="C23" s="15"/>
+      <c r="D23" s="16"/>
+      <c r="E23" s="16"/>
+      <c r="F23" s="16"/>
+      <c r="G23" s="27"/>
+      <c r="H23" s="17"/>
+      <c r="I23" s="17"/>
+      <c r="J23" s="18"/>
+      <c r="K23" s="18"/>
+      <c r="M23" s="19"/>
     </row>
     <row r="24" spans="1:13" ht="19.350000000000001" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A24" s="47">
+      <c r="A24" s="13">
         <f>A23+1</f>
         <v>11</v>
       </c>
-      <c r="B24" s="48" t="str">
+      <c r="B24" s="14" t="str">
         <f t="shared" si="2"/>
         <v>水</v>
       </c>
-      <c r="C24" s="49"/>
-      <c r="D24" s="50"/>
-      <c r="E24" s="50"/>
-      <c r="F24" s="50"/>
-      <c r="G24" s="63"/>
-      <c r="H24" s="51"/>
-      <c r="I24" s="51"/>
-      <c r="J24" s="52"/>
-      <c r="K24" s="52"/>
-      <c r="M24" s="53"/>
+      <c r="C24" s="15"/>
+      <c r="D24" s="16"/>
+      <c r="E24" s="16"/>
+      <c r="F24" s="16"/>
+      <c r="G24" s="27"/>
+      <c r="H24" s="17"/>
+      <c r="I24" s="17"/>
+      <c r="J24" s="18"/>
+      <c r="K24" s="18"/>
+      <c r="M24" s="19"/>
     </row>
     <row r="25" spans="1:13" ht="19.350000000000001" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A25" s="47">
+      <c r="A25" s="13">
         <f>A24+1</f>
         <v>12</v>
       </c>
-      <c r="B25" s="48" t="str">
+      <c r="B25" s="14" t="str">
         <f t="shared" si="2"/>
         <v>木</v>
       </c>
-      <c r="C25" s="49"/>
-      <c r="D25" s="50"/>
-      <c r="E25" s="50"/>
-      <c r="F25" s="50"/>
-      <c r="G25" s="63"/>
-      <c r="H25" s="51"/>
-      <c r="I25" s="51"/>
-      <c r="J25" s="52"/>
-      <c r="K25" s="52"/>
-      <c r="M25" s="53"/>
+      <c r="C25" s="15"/>
+      <c r="D25" s="16"/>
+      <c r="E25" s="16"/>
+      <c r="F25" s="16"/>
+      <c r="G25" s="27"/>
+      <c r="H25" s="17"/>
+      <c r="I25" s="17"/>
+      <c r="J25" s="18"/>
+      <c r="K25" s="18"/>
+      <c r="M25" s="19"/>
     </row>
     <row r="26" spans="1:13" ht="19.350000000000001" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A26" s="47">
+      <c r="A26" s="13">
         <f t="shared" ref="A26:A31" si="3">A25+1</f>
         <v>13</v>
       </c>
-      <c r="B26" s="48" t="str">
+      <c r="B26" s="14" t="str">
         <f t="shared" si="2"/>
         <v>金</v>
       </c>
-      <c r="C26" s="49"/>
-      <c r="D26" s="50"/>
-      <c r="E26" s="50"/>
-      <c r="F26" s="50"/>
-      <c r="G26" s="63"/>
-      <c r="H26" s="51"/>
-      <c r="I26" s="51"/>
-      <c r="J26" s="52"/>
-      <c r="K26" s="52"/>
-      <c r="M26" s="53"/>
+      <c r="C26" s="15"/>
+      <c r="D26" s="16"/>
+      <c r="E26" s="16"/>
+      <c r="F26" s="16"/>
+      <c r="G26" s="27"/>
+      <c r="H26" s="17"/>
+      <c r="I26" s="17"/>
+      <c r="J26" s="18"/>
+      <c r="K26" s="18"/>
+      <c r="M26" s="19"/>
     </row>
     <row r="27" spans="1:13" ht="19.350000000000001" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A27" s="47">
+      <c r="A27" s="13">
         <f t="shared" si="3"/>
         <v>14</v>
       </c>
-      <c r="B27" s="48" t="str">
+      <c r="B27" s="14" t="str">
         <f t="shared" si="2"/>
         <v>土</v>
       </c>
-      <c r="C27" s="49"/>
-      <c r="D27" s="50"/>
-      <c r="E27" s="50"/>
-      <c r="F27" s="50"/>
-      <c r="G27" s="63"/>
-      <c r="H27" s="51"/>
-      <c r="I27" s="51"/>
-      <c r="J27" s="52"/>
-      <c r="K27" s="52"/>
-      <c r="M27" s="53"/>
+      <c r="C27" s="15"/>
+      <c r="D27" s="16"/>
+      <c r="E27" s="16"/>
+      <c r="F27" s="16"/>
+      <c r="G27" s="27"/>
+      <c r="H27" s="17"/>
+      <c r="I27" s="17"/>
+      <c r="J27" s="18"/>
+      <c r="K27" s="18"/>
+      <c r="M27" s="19"/>
     </row>
     <row r="28" spans="1:13" ht="19.350000000000001" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A28" s="47">
+      <c r="A28" s="13">
         <f t="shared" si="3"/>
         <v>15</v>
       </c>
-      <c r="B28" s="48" t="str">
+      <c r="B28" s="14" t="str">
         <f>IF(A28="","",CHOOSE(WEEKDAY(A28),"日","月","火","水","木","金","土"))</f>
         <v>日</v>
       </c>
-      <c r="C28" s="49"/>
-      <c r="D28" s="50"/>
-      <c r="E28" s="50"/>
-      <c r="F28" s="50"/>
-      <c r="G28" s="63"/>
-      <c r="H28" s="51"/>
-      <c r="I28" s="51"/>
-      <c r="J28" s="52"/>
-      <c r="K28" s="52"/>
-      <c r="M28" s="53"/>
+      <c r="C28" s="15"/>
+      <c r="D28" s="16"/>
+      <c r="E28" s="16"/>
+      <c r="F28" s="16"/>
+      <c r="G28" s="27"/>
+      <c r="H28" s="17"/>
+      <c r="I28" s="17"/>
+      <c r="J28" s="18"/>
+      <c r="K28" s="18"/>
+      <c r="M28" s="19"/>
     </row>
     <row r="29" spans="1:13" ht="19.350000000000001" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A29" s="47">
+      <c r="A29" s="13">
         <f t="shared" si="3"/>
         <v>16</v>
       </c>
-      <c r="B29" s="48" t="str">
+      <c r="B29" s="14" t="str">
         <f t="shared" ref="B29:B39" si="4">IF(A29="","",CHOOSE(WEEKDAY(A29),"日","月","火","水","木","金","土"))</f>
         <v>月</v>
       </c>
-      <c r="C29" s="49"/>
-      <c r="D29" s="50"/>
-      <c r="E29" s="50"/>
-      <c r="F29" s="50"/>
-      <c r="G29" s="63"/>
-      <c r="H29" s="51"/>
-      <c r="I29" s="51"/>
-      <c r="J29" s="52"/>
-      <c r="K29" s="52"/>
-      <c r="M29" s="53"/>
+      <c r="C29" s="15"/>
+      <c r="D29" s="16"/>
+      <c r="E29" s="16"/>
+      <c r="F29" s="16"/>
+      <c r="G29" s="27"/>
+      <c r="H29" s="17"/>
+      <c r="I29" s="17"/>
+      <c r="J29" s="18"/>
+      <c r="K29" s="18"/>
+      <c r="M29" s="19"/>
     </row>
     <row r="30" spans="1:13" ht="19.350000000000001" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A30" s="47">
+      <c r="A30" s="13">
         <f t="shared" si="3"/>
         <v>17</v>
       </c>
-      <c r="B30" s="48" t="str">
+      <c r="B30" s="14" t="str">
         <f t="shared" si="4"/>
         <v>火</v>
       </c>
-      <c r="C30" s="49"/>
-      <c r="D30" s="50"/>
-      <c r="E30" s="50"/>
-      <c r="F30" s="50"/>
-      <c r="G30" s="63"/>
-      <c r="H30" s="51"/>
-      <c r="I30" s="51"/>
-      <c r="J30" s="52"/>
-      <c r="K30" s="52"/>
-      <c r="M30" s="53"/>
+      <c r="C30" s="15"/>
+      <c r="D30" s="16"/>
+      <c r="E30" s="16"/>
+      <c r="F30" s="16"/>
+      <c r="G30" s="27"/>
+      <c r="H30" s="17"/>
+      <c r="I30" s="17"/>
+      <c r="J30" s="18"/>
+      <c r="K30" s="18"/>
+      <c r="M30" s="19"/>
     </row>
     <row r="31" spans="1:13" ht="19.350000000000001" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A31" s="47">
+      <c r="A31" s="13">
         <f t="shared" si="3"/>
         <v>18</v>
       </c>
-      <c r="B31" s="48" t="str">
+      <c r="B31" s="14" t="str">
         <f t="shared" si="4"/>
         <v>水</v>
       </c>
-      <c r="C31" s="49"/>
-      <c r="D31" s="50"/>
-      <c r="E31" s="50"/>
-      <c r="F31" s="50"/>
-      <c r="G31" s="63"/>
-      <c r="H31" s="51"/>
-      <c r="I31" s="51"/>
-      <c r="J31" s="52"/>
-      <c r="K31" s="52"/>
-      <c r="M31" s="53"/>
+      <c r="C31" s="15"/>
+      <c r="D31" s="16"/>
+      <c r="E31" s="16"/>
+      <c r="F31" s="16"/>
+      <c r="G31" s="27"/>
+      <c r="H31" s="17"/>
+      <c r="I31" s="17"/>
+      <c r="J31" s="18"/>
+      <c r="K31" s="18"/>
+      <c r="M31" s="19"/>
     </row>
     <row r="32" spans="1:13" ht="19.350000000000001" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A32" s="47">
+      <c r="A32" s="13">
         <f>A31+1</f>
         <v>19</v>
       </c>
-      <c r="B32" s="48" t="str">
+      <c r="B32" s="14" t="str">
         <f t="shared" si="4"/>
         <v>木</v>
       </c>
-      <c r="C32" s="49"/>
-      <c r="D32" s="50"/>
-      <c r="E32" s="50"/>
-      <c r="F32" s="50"/>
-      <c r="G32" s="63"/>
-      <c r="H32" s="51"/>
-      <c r="I32" s="51"/>
-      <c r="J32" s="52"/>
-      <c r="K32" s="52"/>
-      <c r="M32" s="53"/>
+      <c r="C32" s="15"/>
+      <c r="D32" s="16"/>
+      <c r="E32" s="16"/>
+      <c r="F32" s="16"/>
+      <c r="G32" s="27"/>
+      <c r="H32" s="17"/>
+      <c r="I32" s="17"/>
+      <c r="J32" s="18"/>
+      <c r="K32" s="18"/>
+      <c r="M32" s="19"/>
     </row>
     <row r="33" spans="1:13" ht="19.350000000000001" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A33" s="47">
+      <c r="A33" s="13">
         <f>A32+1</f>
         <v>20</v>
       </c>
-      <c r="B33" s="48" t="str">
+      <c r="B33" s="14" t="str">
         <f t="shared" si="4"/>
         <v>金</v>
       </c>
-      <c r="C33" s="49"/>
-      <c r="D33" s="50"/>
-      <c r="E33" s="50"/>
-      <c r="F33" s="50"/>
-      <c r="G33" s="63"/>
-      <c r="H33" s="51"/>
-      <c r="I33" s="51"/>
-      <c r="J33" s="52"/>
-      <c r="K33" s="52"/>
-      <c r="M33" s="53"/>
+      <c r="C33" s="15"/>
+      <c r="D33" s="16"/>
+      <c r="E33" s="16"/>
+      <c r="F33" s="16"/>
+      <c r="G33" s="27"/>
+      <c r="H33" s="17"/>
+      <c r="I33" s="17"/>
+      <c r="J33" s="18"/>
+      <c r="K33" s="18"/>
+      <c r="M33" s="19"/>
     </row>
     <row r="34" spans="1:13" ht="19.350000000000001" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A34" s="47">
+      <c r="A34" s="13">
         <f t="shared" ref="A34:A35" si="5">A33+1</f>
         <v>21</v>
       </c>
-      <c r="B34" s="48" t="str">
+      <c r="B34" s="14" t="str">
         <f t="shared" si="4"/>
         <v>土</v>
       </c>
-      <c r="C34" s="49"/>
-      <c r="D34" s="50"/>
-      <c r="E34" s="50"/>
-      <c r="F34" s="50"/>
-      <c r="G34" s="63"/>
-      <c r="H34" s="51"/>
-      <c r="I34" s="51"/>
-      <c r="J34" s="52"/>
-      <c r="K34" s="52"/>
-      <c r="M34" s="53"/>
+      <c r="C34" s="15"/>
+      <c r="D34" s="16"/>
+      <c r="E34" s="16"/>
+      <c r="F34" s="16"/>
+      <c r="G34" s="27"/>
+      <c r="H34" s="17"/>
+      <c r="I34" s="17"/>
+      <c r="J34" s="18"/>
+      <c r="K34" s="18"/>
+      <c r="M34" s="19"/>
     </row>
     <row r="35" spans="1:13" ht="19.350000000000001" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A35" s="47">
+      <c r="A35" s="13">
         <f t="shared" si="5"/>
         <v>22</v>
       </c>
-      <c r="B35" s="48" t="str">
+      <c r="B35" s="14" t="str">
         <f t="shared" si="4"/>
         <v>日</v>
       </c>
-      <c r="C35" s="49"/>
-      <c r="D35" s="50"/>
-      <c r="E35" s="50"/>
-      <c r="F35" s="50"/>
-      <c r="G35" s="63"/>
-      <c r="H35" s="51"/>
-      <c r="I35" s="51"/>
-      <c r="J35" s="52"/>
-      <c r="K35" s="52"/>
-      <c r="M35" s="53"/>
+      <c r="C35" s="15"/>
+      <c r="D35" s="16"/>
+      <c r="E35" s="16"/>
+      <c r="F35" s="16"/>
+      <c r="G35" s="27"/>
+      <c r="H35" s="17"/>
+      <c r="I35" s="17"/>
+      <c r="J35" s="18"/>
+      <c r="K35" s="18"/>
+      <c r="M35" s="19"/>
     </row>
     <row r="36" spans="1:13" ht="19.350000000000001" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A36" s="47">
+      <c r="A36" s="13">
         <f>A35+1</f>
         <v>23</v>
       </c>
-      <c r="B36" s="48" t="str">
+      <c r="B36" s="14" t="str">
         <f t="shared" si="4"/>
         <v>月</v>
       </c>
-      <c r="C36" s="49"/>
-      <c r="D36" s="50"/>
-      <c r="E36" s="50"/>
-      <c r="F36" s="50"/>
-      <c r="G36" s="63"/>
-      <c r="H36" s="51"/>
-      <c r="I36" s="51"/>
-      <c r="J36" s="52"/>
-      <c r="K36" s="52"/>
-      <c r="M36" s="53"/>
+      <c r="C36" s="15"/>
+      <c r="D36" s="16"/>
+      <c r="E36" s="16"/>
+      <c r="F36" s="16"/>
+      <c r="G36" s="27"/>
+      <c r="H36" s="17"/>
+      <c r="I36" s="17"/>
+      <c r="J36" s="18"/>
+      <c r="K36" s="18"/>
+      <c r="M36" s="19"/>
     </row>
     <row r="37" spans="1:13" ht="19.350000000000001" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A37" s="47">
+      <c r="A37" s="13">
         <f>A36+1</f>
         <v>24</v>
       </c>
-      <c r="B37" s="48" t="str">
+      <c r="B37" s="14" t="str">
         <f t="shared" si="4"/>
         <v>火</v>
       </c>
-      <c r="C37" s="49"/>
-      <c r="D37" s="50"/>
-      <c r="E37" s="50"/>
-      <c r="F37" s="50"/>
-      <c r="G37" s="63"/>
-      <c r="H37" s="51"/>
-      <c r="I37" s="51"/>
-      <c r="J37" s="52"/>
-      <c r="K37" s="52"/>
-      <c r="M37" s="53"/>
+      <c r="C37" s="15"/>
+      <c r="D37" s="16"/>
+      <c r="E37" s="16"/>
+      <c r="F37" s="16"/>
+      <c r="G37" s="27"/>
+      <c r="H37" s="17"/>
+      <c r="I37" s="17"/>
+      <c r="J37" s="18"/>
+      <c r="K37" s="18"/>
+      <c r="M37" s="19"/>
     </row>
     <row r="38" spans="1:13" ht="19.350000000000001" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A38" s="47">
+      <c r="A38" s="13">
         <f>A37+1</f>
         <v>25</v>
       </c>
-      <c r="B38" s="48" t="str">
+      <c r="B38" s="14" t="str">
         <f t="shared" si="4"/>
         <v>水</v>
       </c>
-      <c r="C38" s="49"/>
-      <c r="D38" s="50"/>
-      <c r="E38" s="50"/>
-      <c r="F38" s="50"/>
-      <c r="G38" s="63"/>
-      <c r="H38" s="51"/>
-      <c r="I38" s="51"/>
-      <c r="J38" s="52"/>
-      <c r="K38" s="52"/>
-      <c r="M38" s="53"/>
+      <c r="C38" s="15"/>
+      <c r="D38" s="16"/>
+      <c r="E38" s="16"/>
+      <c r="F38" s="16"/>
+      <c r="G38" s="27"/>
+      <c r="H38" s="17"/>
+      <c r="I38" s="17"/>
+      <c r="J38" s="18"/>
+      <c r="K38" s="18"/>
+      <c r="M38" s="19"/>
     </row>
     <row r="39" spans="1:13" ht="19.350000000000001" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A39" s="47">
+      <c r="A39" s="13">
         <f>A38+1</f>
         <v>26</v>
       </c>
-      <c r="B39" s="48" t="str">
+      <c r="B39" s="14" t="str">
         <f t="shared" si="4"/>
         <v>木</v>
       </c>
-      <c r="C39" s="49"/>
-      <c r="D39" s="50"/>
-      <c r="E39" s="50"/>
-      <c r="F39" s="50"/>
-      <c r="G39" s="63"/>
-      <c r="H39" s="51"/>
-      <c r="I39" s="51"/>
-      <c r="J39" s="52"/>
-      <c r="K39" s="52"/>
-      <c r="M39" s="53"/>
+      <c r="C39" s="15"/>
+      <c r="D39" s="16"/>
+      <c r="E39" s="16"/>
+      <c r="F39" s="16"/>
+      <c r="G39" s="27"/>
+      <c r="H39" s="17"/>
+      <c r="I39" s="17"/>
+      <c r="J39" s="18"/>
+      <c r="K39" s="18"/>
+      <c r="M39" s="19"/>
     </row>
     <row r="40" spans="1:13" ht="19.350000000000001" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A40" s="47">
+      <c r="A40" s="13">
         <f t="shared" ref="A40:A41" si="6">A39+1</f>
         <v>27</v>
       </c>
-      <c r="B40" s="48" t="str">
+      <c r="B40" s="14" t="str">
         <f t="shared" ref="B40:B43" si="7">IF(A40="","",CHOOSE(WEEKDAY(A40),"日","月","火","水","木","金","土"))</f>
         <v>金</v>
       </c>
-      <c r="C40" s="49"/>
-      <c r="D40" s="50"/>
-      <c r="E40" s="50"/>
-      <c r="F40" s="50"/>
-      <c r="G40" s="63"/>
-      <c r="H40" s="51"/>
-      <c r="I40" s="51"/>
-      <c r="J40" s="52"/>
-      <c r="K40" s="52"/>
-      <c r="M40" s="53"/>
+      <c r="C40" s="15"/>
+      <c r="D40" s="16"/>
+      <c r="E40" s="16"/>
+      <c r="F40" s="16"/>
+      <c r="G40" s="27"/>
+      <c r="H40" s="17"/>
+      <c r="I40" s="17"/>
+      <c r="J40" s="18"/>
+      <c r="K40" s="18"/>
+      <c r="M40" s="19"/>
     </row>
     <row r="41" spans="1:13" ht="19.350000000000001" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A41" s="47">
+      <c r="A41" s="13">
         <f t="shared" si="6"/>
         <v>28</v>
       </c>
-      <c r="B41" s="48" t="str">
+      <c r="B41" s="14" t="str">
         <f t="shared" si="7"/>
         <v>土</v>
       </c>
-      <c r="C41" s="49"/>
-      <c r="D41" s="50"/>
-      <c r="E41" s="50"/>
-      <c r="F41" s="50"/>
-      <c r="G41" s="63"/>
-      <c r="H41" s="51"/>
-      <c r="I41" s="51"/>
-      <c r="J41" s="52"/>
-      <c r="K41" s="52"/>
-      <c r="M41" s="53"/>
+      <c r="C41" s="15"/>
+      <c r="D41" s="16"/>
+      <c r="E41" s="16"/>
+      <c r="F41" s="16"/>
+      <c r="G41" s="27"/>
+      <c r="H41" s="17"/>
+      <c r="I41" s="17"/>
+      <c r="J41" s="18"/>
+      <c r="K41" s="18"/>
+      <c r="M41" s="19"/>
     </row>
     <row r="42" spans="1:13" ht="19.350000000000001" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A42" s="47">
+      <c r="A42" s="13">
         <f>A41+1</f>
         <v>29</v>
       </c>
-      <c r="B42" s="48" t="str">
+      <c r="B42" s="14" t="str">
         <f t="shared" si="7"/>
         <v>日</v>
       </c>
-      <c r="C42" s="49"/>
-      <c r="D42" s="50"/>
-      <c r="E42" s="50"/>
-      <c r="F42" s="50"/>
-      <c r="G42" s="64"/>
-      <c r="H42" s="51"/>
-      <c r="I42" s="51"/>
-      <c r="J42" s="52"/>
-      <c r="K42" s="52"/>
-      <c r="M42" s="53"/>
+      <c r="C42" s="15"/>
+      <c r="D42" s="16"/>
+      <c r="E42" s="16"/>
+      <c r="F42" s="16"/>
+      <c r="G42" s="28"/>
+      <c r="H42" s="17"/>
+      <c r="I42" s="17"/>
+      <c r="J42" s="18"/>
+      <c r="K42" s="18"/>
+      <c r="M42" s="19"/>
     </row>
     <row r="43" spans="1:13" ht="19.350000000000001" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A43" s="47">
+      <c r="A43" s="13">
         <f>A42+1</f>
         <v>30</v>
       </c>
-      <c r="B43" s="48" t="str">
+      <c r="B43" s="14" t="str">
         <f t="shared" si="7"/>
         <v>月</v>
       </c>
-      <c r="C43" s="49"/>
-      <c r="D43" s="50"/>
-      <c r="E43" s="50"/>
-      <c r="F43" s="50"/>
-      <c r="G43" s="64"/>
-      <c r="H43" s="51"/>
-      <c r="I43" s="51"/>
-      <c r="J43" s="52"/>
-      <c r="K43" s="52"/>
-      <c r="M43" s="53"/>
+      <c r="C43" s="15"/>
+      <c r="D43" s="16"/>
+      <c r="E43" s="16"/>
+      <c r="F43" s="16"/>
+      <c r="G43" s="28"/>
+      <c r="H43" s="17"/>
+      <c r="I43" s="17"/>
+      <c r="J43" s="18"/>
+      <c r="K43" s="18"/>
+      <c r="M43" s="19"/>
     </row>
     <row r="44" spans="1:13" ht="19.350000000000001" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A44" s="54" t="s">
+      <c r="A44" s="29" t="s">
         <v>23</v>
       </c>
-      <c r="B44" s="55"/>
-      <c r="C44" s="56">
+      <c r="B44" s="30"/>
+      <c r="C44" s="20">
         <f>COUNTA(H13:H43)</f>
         <v>0</v>
       </c>
-      <c r="D44" s="57" t="s">
+      <c r="D44" s="21" t="s">
         <v>15</v>
       </c>
-      <c r="E44" s="58" t="s">
+      <c r="E44" s="22" t="s">
         <v>22</v>
       </c>
-      <c r="F44" s="59">
+      <c r="F44" s="23">
         <f>(SUM(K13:K43)/TIME(1,,))</f>
         <v>0</v>
       </c>
-      <c r="G44" s="57" t="s">
+      <c r="G44" s="21" t="s">
         <v>24</v>
       </c>
-      <c r="H44" s="58" t="s">
+      <c r="H44" s="22" t="s">
         <v>25</v>
       </c>
-      <c r="I44" s="60">
-        <f>$F$44-$C$44*8</f>
+      <c r="I44" s="24">
+        <f>MAX(0, $F$44 - $C$44 * "8:00")</f>
         <v>0</v>
       </c>
-      <c r="J44" s="61" t="s">
+      <c r="J44" s="25" t="s">
         <v>24</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="20">
+    <mergeCell ref="A2:H2"/>
+    <mergeCell ref="I2:K2"/>
+    <mergeCell ref="A3:C3"/>
+    <mergeCell ref="D3:H3"/>
+    <mergeCell ref="A4:C4"/>
+    <mergeCell ref="D4:H4"/>
     <mergeCell ref="A44:B44"/>
     <mergeCell ref="A5:C5"/>
     <mergeCell ref="D5:H5"/>
@@ -1844,12 +1850,6 @@
     <mergeCell ref="G9:H9"/>
     <mergeCell ref="A10:C10"/>
     <mergeCell ref="D10:H10"/>
-    <mergeCell ref="A2:H2"/>
-    <mergeCell ref="I2:K2"/>
-    <mergeCell ref="A3:C3"/>
-    <mergeCell ref="D3:H3"/>
-    <mergeCell ref="A4:C4"/>
-    <mergeCell ref="D4:H4"/>
   </mergeCells>
   <phoneticPr fontId="3"/>
   <printOptions horizontalCentered="1"/>
@@ -1873,15 +1873,6 @@
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100DC957A2BAE3FEB488DD90F3CEEBA64B2" ma:contentTypeVersion="12" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="5f1653939578ce63f276984d74f7b80f">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="fddd5c7a-2dc9-4280-9104-0c5c090f8913" xmlns:ns3="49da8719-5195-4d58-b9e3-040d669e384e" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="31f706c199e200b5ceeaeb3f8c022435" ns2:_="" ns3:_="">
     <xsd:import namespace="fddd5c7a-2dc9-4280-9104-0c5c090f8913"/>
@@ -2082,6 +2073,15 @@
 </ct:contentTypeSchema>
 </file>
 
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{A7A8AE5A-FCD2-4F3B-B711-AC3CFBE815ED}">
   <ds:schemaRefs>
@@ -2095,14 +2095,6 @@
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{F9C41F5C-CAF1-47CB-985C-96AFA693AEFA}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{27D2DB86-FB68-473C-AC36-38170BDA1492}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -2119,4 +2111,12 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{F9C41F5C-CAF1-47CB-985C-96AFA693AEFA}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
</xml_diff>